<commit_message>
Updated composition: 77.3% field completion, 0.36 avg confidence, zero non-US/EU records. Regenerated the CSV/XLSX export to match
</commit_message>
<xml_diff>
--- a/data/family_office_dataset.xlsx
+++ b/data/family_office_dataset.xlsx
@@ -583,22 +583,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Adar Poonawalla Family Office</t>
+          <t>Allie Family Office LLC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Single-Family Office</t>
+          <t>Multi-Family Office</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Adar Poonawalla (father Cyrus Poonawalla)</t>
+          <t>Bruno Ghio</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CEO, Serum Institute of India</t>
+          <t>Sole Owner</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -606,48 +606,60 @@
         <v>0</v>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/bruno-ghio-1264b616b/</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://allie-intl.com</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Pune</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Family wealth ~$15B (not a precise AUM figure)</t>
+          <t>~$1.15B as of Dec 31, 2024 ($508.69M discretionary, $637.88M limited discretionary)</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Diversified beyond the family's core vaccine/pharma business into financial services (NBFC lending), renewable energy, and real estate - strategically positioned around India's expanding financial-services market and clean-energy transition.</t>
+          <t>Long-term wealth preservation with strategic asset allocation and jurisdiction diversification (to mitigate country risk) - relevant for Latin American families managing cross-border wealth. Diversifies into direct assets, ETFs, and specialized funds; customized benchmarks and periodic reporting per client.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Consumer, life sciences, financial services (commercial/agri/SME/mortgage finance, insurance - rural/semi-urban focus), clean/renewable energy, real estate</t>
+          <t>Direct assets, ETFs, specialized funds - diversified by jurisdiction</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Invests mainly through Rising Sun Holdings, the Cyrus Poonawalla Group's investment holding company (incorporated 1993). Serum Institute (founded 1966) is the world's largest vaccine maker by doses.</t>
+          <t>Founded September 2019. Focuses on Peruvian and broader Latin American HNW families and multi-generational family governance.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Invested Rs 700 crore (~$84M) in Inox Clean Energy.</t>
+          <t>Most recent 13F filing (2026-05-14) shows a position in Spdr S&amp;P 500 Etf Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="T2" t="b">
@@ -655,20 +667,20 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>India (Pune). Manages the wealth of Adar Poonawalla, CEO of Serum Institute of India (world's largest vaccine maker). Invests mainly through 'Rising Sun Holdings', the Cyrus Poonawalla Group's investment holding company (incorporated 1993) - these are the SAME family's vehicle, not two separate entities (a second raw candidate 'Rising Sun Holdings' from the same discovery run refers to this). Family wealth ~$15B. Multiply corroborated: familyofficehub.io, PipelineRoad, Wikipedia.</t>
+          <t>Founded 2019 by Bruno Ghio (sole owner), serves multiple Latin American/Peruvian HNW families, $1.15B AUM. Third-party source explicitly labels it 'Miami Multi Family Office'.</t>
         </is>
       </c>
       <c r="V2" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>multi_source_corroboration</t>
+          <t>third_party_directory</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>multi_source_corroboration: https://pipelineroad.com/directory/poonawalla-family</t>
+          <t>third_party_directory: https://altss.com/profile/alli-family-office-llc</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -678,29 +690,29 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Foreign entity (India) - press/database verified, not SEC-primary verified.</t>
+          <t>CAVEAT: multi-family classification rests only on a secondary aggregator label (e.g. Altss), not a primary quote from the firm itself. Not independently confirmed - same source class that was WRONG for Family Manage LLC (Altss said single-family, firm site said multi-family). Lower confidence than other MFO records in this file. Recommend a direct-site check before treating as equally solid. | 13F-HR filer, matched keyword 'family office'. Location: Miami, FL. | Personal email explicitly noted as available only via paid aggregator subscription, not in public results - left blank rather than guess.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Allie Family Office LLC</t>
+          <t>Appaloosa Management</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Multi-Family Office</t>
+          <t>Single-Family Office</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bruno Ghio</t>
+          <t>David Tepper</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sole Owner</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -708,20 +720,20 @@
         <v>0</v>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/bruno-ghio-1264b616b/</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/appaloosa-management-lp</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://allie-intl.com</t>
+          <t>https://www.amlp.com</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Beach</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -734,34 +746,30 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>~$1.15B as of Dec 31, 2024 ($508.69M discretionary, $637.88M limited discretionary)</t>
-        </is>
-      </c>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Long-term wealth preservation with strategic asset allocation and jurisdiction diversification (to mitigate country risk) - relevant for Latin American families managing cross-border wealth. Diversifies into direct assets, ETFs, and specialized funds; customized benchmarks and periodic reporting per client.</t>
+          <t>Public equities with sector conviction (e.g. tripled Micron stake in Q1 2026 on semiconductor demand); continues Tepper's macro/distressed-credit-informed public markets approach from his hedge fund era.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Direct assets, ETFs, specialized funds - diversified by jurisdiction</t>
+          <t>Public equities, semiconductor/technology conviction positions</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Founded September 2019. Focuses on Peruvian and broader Latin American HNW families and multi-generational family governance.</t>
+          <t>Converted from a $13B hedge fund to a pure family office in 2019, returning outside investor capital. Manages Tepper's personal ~$15B fortune.</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-05-14) shows a position in Spdr S&amp;P 500 Etf Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+          <t>Tripled Micron position to $428.1M in Q1 2026.</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="T3" t="b">
@@ -769,20 +777,20 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Founded 2019 by Bruno Ghio (sole owner), serves multiple Latin American/Peruvian HNW families, $1.15B AUM. Third-party source explicitly labels it 'Miami Multi Family Office'.</t>
+          <t>Short Hills, NJ. Converted from a $13B hedge fund to a pure family office in 2019 - returned essentially all outside investor capital (exiting investors received 90% back Jan 2020, rest by Apr 2020), now manages Tepper's personal ~$15B fortune exclusively. CNBC headline directly: 'David Tepper converting hedge fund into family office, returning outside capital.' Confirmed current/recent activity: tripled Micron position to $428.1M per 2026 Q1 CNBC coverage.</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0.1</v>
+        <v>0.65</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>third_party_directory</t>
+          <t>press_named_sfo, multi_source_corroboration</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>third_party_directory: https://altss.com/profile/alli-family-office-llc</t>
+          <t>press_named_sfo: https://www.cnbc.com/2019/05/23/david-tepper-is-reportedly-converting-hedge-fund-into-a-family-office-returning-outside-capital.html | multi_source_corroboration: https://www.cnbc.com/2026/05/21/billionaire-investments-q1.html</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -792,55 +800,63 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>CAVEAT: multi-family classification rests only on a secondary aggregator label (e.g. Altss), not a primary quote from the firm itself. Not independently confirmed - same source class that was WRONG for Family Manage LLC (Altss said single-family, firm site said multi-family). Lower confidence than other MFO records in this file. Recommend a direct-site check before treating as equally solid. | 13F-HR filer, matched keyword 'family office'. Location: Miami, FL. | Personal email explicitly noted as available only via paid aggregator subscription, not in public results - left blank rather than guess.</t>
+          <t>Press/database verified (CNBC, Forbes, Institutional Investor), not SEC-primary verified. | Relocated from Chatham, NJ (original 1993 HQ) to Miami Beach, FL in 2016. | Corporate LinkedIn confirmed via web search - official company page for the firm (financial services category), name matches exactly. A candidate personal LinkedIn for David Tepper was also found but NOT added - insufficient time to independently verify authenticity given high impersonation risk for public figures.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Appaloosa Management</t>
+          <t>Arrowroot Family Office, LLC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Single-Family Office</t>
+          <t>Multi-Family Office</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>David Tepper</t>
+          <t>Rob Santos</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>CEO / Principal Owner</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="b">
         <v>0</v>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>+1 310-341-4774</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rob-santos-afo/</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/appaloosa-management-lp</t>
+          <t>https://www.linkedin.com/company/arrowroot-family-office</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.amlp.com</t>
+          <t>https://arrowrootfamilyoffice.com</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Miami Beach</t>
+          <t>Marina del Rey</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -848,30 +864,34 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>$373.9M-$431M (varies by source/reporting date)</t>
+        </is>
+      </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Public equities with sector conviction (e.g. tripled Micron stake in Q1 2026 on semiconductor demand); continues Tepper's macro/distressed-credit-informed public markets approach from his hedge fund era.</t>
+          <t>Fiduciary-only approach: no proprietary products, open architecture, conflict-free ('only incentive is client outcome'). Data-driven, focused on multigenerational wealth retention; integrated team of advisors, accountants, and lawyers.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Public equities, semiconductor/technology conviction positions</t>
+          <t>Diversified public/private portfolios via open-architecture implementation</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Converted from a $13B hedge fund to a pure family office in 2019, returning outside investor capital. Manages Tepper's personal ~$15B fortune.</t>
+          <t>Founded 2013 as 'Vitreous Partners' by ex-investment banker Rob Santos, rebranded 2017. ~18 employees.</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Tripled Micron position to $428.1M in Q1 2026.</t>
+          <t>Most recent 13F filing (2026-05-14) shows a position in Vanguard Scottsdale Fds. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="T4" t="b">
@@ -879,20 +899,20 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Short Hills, NJ. Converted from a $13B hedge fund to a pure family office in 2019 - returned essentially all outside investor capital (exiting investors received 90% back Jan 2020, rest by Apr 2020), now manages Tepper's personal ~$15B fortune exclusively. CNBC headline directly: 'David Tepper converting hedge fund into family office, returning outside capital.' Confirmed current/recent activity: tripled Micron position to $428.1M per 2026 Q1 CNBC coverage.</t>
+          <t>Founded 2013 by Rob Santos (ex-investment banker, not family money), rebranded from 'Vitreous Partners' 2017, explicitly serves 'affluent families, entrepreneurs, individuals, trusts, estates, charitable organizations' - plural client base, RIA model.</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>0.65</v>
+        <v>0.25</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>press_named_sfo, multi_source_corroboration</t>
+          <t>own_website</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.cnbc.com/2019/05/23/david-tepper-is-reportedly-converting-hedge-fund-into-a-family-office-returning-outside-capital.html | multi_source_corroboration: https://www.cnbc.com/2026/05/21/billionaire-investments-q1.html</t>
+          <t>own_website: https://arrowrootfamilyoffice.com/about/</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -902,14 +922,14 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>Press/database verified (CNBC, Forbes, Institutional Investor), not SEC-primary verified. | Relocated from Chatham, NJ (original 1993 HQ) to Miami Beach, FL in 2016. | Corporate LinkedIn confirmed via web search - official company page for the firm (financial services category), name matches exactly. A candidate personal LinkedIn for David Tepper was also found but NOT added - insufficient time to independently verify authenticity given high impersonation risk for public figures.</t>
+          <t>13F-HR filer, matched keyword 'family office'. Location: Marina Del Rey, CA. | Aggregator sites (ContactOut/RocketReach) list 4 CONFLICTING candidate emails across different domains (arrowrootpartners.com, arrowrootadvisors.com, arrowrootfamilyoffice.com, plus a personal gmail) - could not determine the current authoritative address, left principal_email blank rather than guess. Phone/LinkedIn are single-source, lower risk.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Arrowroot Family Office, LLC</t>
+          <t>Avantra Family Wealth, Inc.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -919,46 +939,50 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Rob Santos</t>
+          <t>Kim Kenawell</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CEO / Principal Owner</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>Founder &amp; CEO / Senior Wealth Advisor</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Kim_Kenawell@avantrafamilywealth.com</t>
+        </is>
+      </c>
       <c r="F5" t="b">
         <v>0</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>+1 310-341-4774</t>
+          <t>717-276-1504</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/rob-santos-afo/</t>
+          <t>https://www.linkedin.com/in/kim-lee-kenawell-msfs-abfp-awma-cdfa-crpc-b9905431/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/arrowroot-family-office</t>
+          <t>https://www.linkedin.com/company/avantra-family-wealth</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://arrowrootfamilyoffice.com</t>
+          <t>https://www.avantrafamilywealth.com</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Marina del Rey</t>
+          <t>Mechanicsburg</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -968,32 +992,32 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>$373.9M-$431M (varies by source/reporting date)</t>
+          <t>$194.4M across 990 accounts (967 discretionary, 23 non-discretionary)</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Fiduciary-only approach: no proprietary products, open architecture, conflict-free ('only incentive is client outcome'). Data-driven, focused on multigenerational wealth retention; integrated team of advisors, accountants, and lawyers.</t>
+          <t>Comprehensive, discretionary and non-discretionary portfolio management integrated with financial planning - income generation, retirement, healthcare-cost, and tax-minimization planning - reflecting a concierge, whole-life-wealth approach rather than a narrow asset-allocation-only mandate.</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Diversified public/private portfolios via open-architecture implementation</t>
+          <t>Diversified wealth management - no distinct industry-sector tilt identified</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Founded 2013 as 'Vitreous Partners' by ex-investment banker Rob Santos, rebranded 2017. ~18 employees.</t>
+          <t>Independent, concierge-style multifamily office founded 2017 by Kim Kenawell (Mechanicsburg, PA), serving the HNW community with 30+ years of combined advisory experience.</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-05-14) shows a position in Vanguard Scottsdale Fds. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+          <t>Most recent 13F filing (2026-04-22) shows a position in Apple Inc. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="T5" t="b">
@@ -1001,7 +1025,7 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Founded 2013 by Rob Santos (ex-investment banker, not family money), rebranded from 'Vitreous Partners' 2017, explicitly serves 'affluent families, entrepreneurs, individuals, trusts, estates, charitable organizations' - plural client base, RIA model.</t>
+          <t>Self-described 'concierge-style multifamily office', 990 client accounts, founder Kim Kenawell. Explicit self-declaration as multi-family.</t>
         </is>
       </c>
       <c r="V5" t="n">
@@ -1014,7 +1038,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>own_website: https://arrowrootfamilyoffice.com/about/</t>
+          <t>own_website: https://www.avantrafamilywealth.com/</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -1024,14 +1048,14 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>13F-HR filer, matched keyword 'family office'. Location: Marina Del Rey, CA. | Aggregator sites (ContactOut/RocketReach) list 4 CONFLICTING candidate emails across different domains (arrowrootpartners.com, arrowrootadvisors.com, arrowrootfamilyoffice.com, plus a personal gmail) - could not determine the current authoritative address, left principal_email blank rather than guess. Phone/LinkedIn are single-source, lower risk.</t>
+          <t>13F-HR filer, matched keyword 'family wealth'. Location: Mechanicsburg, PA. | Email matches firm domain from a single consistent source (firm bio page) - not deliverability-confirmed, hence principal_email_verified=False.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Avantra Family Wealth, Inc.</t>
+          <t>BOSTON FAMILY OFFICE LLC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1041,50 +1065,42 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kim Kenawell</t>
+          <t>George Putnam III, George Beal</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Founder &amp; CEO / Senior Wealth Advisor</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Kim_Kenawell@avantrafamilywealth.com</t>
-        </is>
-      </c>
+          <t>Founding Partners</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="b">
         <v>0</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>717-276-1504</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/kim-lee-kenawell-msfs-abfp-awma-cdfa-crpc-b9905431/</t>
-        </is>
-      </c>
+          <t>617-624-0800 (firm main line)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/avantra-family-wealth</t>
+          <t>https://www.linkedin.com/company/boston-family-advisors-llc</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.avantrafamilywealth.com</t>
+          <t>https://www.bosfam.com</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Mechanicsburg</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1094,32 +1110,32 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>$194.4M across 990 accounts (967 discretionary, 23 non-discretionary)</t>
+          <t>$1.87B</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Comprehensive, discretionary and non-discretionary portfolio management integrated with financial planning - income generation, retirement, healthcare-cost, and tax-minimization planning - reflecting a concierge, whole-life-wealth approach rather than a narrow asset-allocation-only mandate.</t>
+          <t>Growth-oriented equities benefiting from favorable macro trends, strong product/service franchises, and good management, balanced with fixed income and other asset classes. Each portfolio manager follows a specific economic sector; diversification maintained via sector-weight and position-size limits.</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Diversified wealth management - no distinct industry-sector tilt identified</t>
+          <t>Growth equities across sectors, plus real estate partnerships, hedge funds, private equity, venture capital as appropriate</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Independent, concierge-style multifamily office founded 2017 by Kim Kenawell (Mechanicsburg, PA), serving the HNW community with 30+ years of combined advisory experience.</t>
+          <t>Founded 1996 by a group including David Richardson Jr., George Putnam III, Ned Weld, Dick Macklem, George Beal, and Solange Bell. Descendants of the Putnam and Richardson families remain involved alongside other partners.</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-04-22) shows a position in Apple Inc. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+          <t>Most recent 13F filing (2026-05-13) top holding: Apple Inc., $72,822k.</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="T6" t="b">
@@ -1127,7 +1143,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Self-described 'concierge-style multifamily office', 990 client accounts, founder Kim Kenawell. Explicit self-declaration as multi-family.</t>
+          <t>Founded 1996 by 6 unrelated principals (Putnam, Richardson, Weld, Macklem, Beal, Bell), $1.87B AUM, ownership distributed (no single family controls &gt;30%), serves 'additional client capital' beyond founders. Explicitly documented as multi-family.</t>
         </is>
       </c>
       <c r="V6" t="n">
@@ -1140,7 +1156,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>own_website: https://www.avantrafamilywealth.com/</t>
+          <t>own_website: https://www.bosfam.com/history/</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1150,59 +1166,51 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>13F-HR filer, matched keyword 'family wealth'. Location: Mechanicsburg, PA. | Email matches firm domain from a single consistent source (firm bio page) - not deliverability-confirmed, hence principal_email_verified=False.</t>
+          <t>13F-HR filer, matched keyword 'family office'. Location: Boston, MA. | CAVEAT: the LinkedIn page found is titled 'Boston Family Advisors, LLC' not 'Boston Family Office LLC' - could be an alternate/prior name for the same entity or a related-but-distinct one. Kept but flagged as unconfirmed exact match. | CAVEAT: Yelp lists this physical location (88 Broad Street) as 'CLOSED - Updated May 2025'. Could indicate a relocation or an actual closure - not resolved with available sources. Worth a direct check before relying on this as a currently operating office.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BOSTON FAMILY OFFICE LLC</t>
+          <t>Bezos Expeditions</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Multi-Family Office</t>
+          <t>Single-Family Office</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>George Putnam III, George Beal</t>
+          <t>Jeff Bezos</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Founding Partners</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="b">
         <v>0</v>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>617-624-0800 (firm main line)</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/boston-family-advisors-llc</t>
-        </is>
-      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.bosfam.com</t>
+          <t>https://www.bezosexpeditions.com</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Mercer Island</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1210,34 +1218,30 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>$1.87B</t>
-        </is>
-      </c>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Growth-oriented equities benefiting from favorable macro trends, strong product/service franchises, and good management, balanced with fixed income and other asset classes. Each portfolio manager follows a specific economic sector; diversification maintained via sector-weight and position-size limits.</t>
+          <t>Founder-investor philosophy prioritizing transformative companies pursuing large market opportunities; willing to hold for very long time horizons. Favors direct founder relationships over intermediary fund managers.</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Growth equities across sectors, plus real estate partnerships, hedge funds, private equity, venture capital as appropriate</t>
+          <t>Biotech, fintech, AI/robotics, space/aerospace, media, real estate, logistics, healthcare, education</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Founded 1996 by a group including David Richardson Jr., George Putnam III, Ned Weld, Dick Macklem, George Beal, and Solange Bell. Descendants of the Putnam and Richardson families remain involved alongside other partners.</t>
+          <t>Jeff Bezos's personal investment vehicle, based on Mercer Island, WA. Backs transformative companies across biotech, fintech, AI/robotics, space, media, real estate, logistics, healthcare, and education.</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-05-13) top holding: Apple Inc., $72,822k.</t>
+          <t>Backed Unconventional AI and Physical Intelligence; ranked #2 in CNBC's 2026 Family Office 15. Backed five AI startups in June 2026 per separate CNBC coverage.</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="T7" t="b">
@@ -1245,74 +1249,90 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Founded 1996 by 6 unrelated principals (Putnam, Richardson, Weld, Macklem, Beal, Bell), $1.87B AUM, ownership distributed (no single family controls &gt;30%), serves 'additional client capital' beyond founders. Explicitly documented as multi-family.</t>
+          <t>Backed Unconventional AI, Physical Intelligence; ranked #2 in CNBC's 2026 list.</t>
         </is>
       </c>
       <c r="V7" t="n">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>own_website</t>
+          <t>press_named_sfo</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>own_website: https://www.bosfam.com/history/</t>
+          <t>press_named_sfo: https://www.cnbc.com/2026/02/12/inside-wealth-family-office-15.html</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>13F-HR filer, matched keyword 'family office'. Location: Boston, MA. | CAVEAT: the LinkedIn page found is titled 'Boston Family Advisors, LLC' not 'Boston Family Office LLC' - could be an alternate/prior name for the same entity or a related-but-distinct one. Kept but flagged as unconfirmed exact match. | CAVEAT: Yelp lists this physical location (88 Broad Street) as 'CLOSED - Updated May 2025'. Could indicate a relocation or an actual closure - not resolved with available sources. Worth a direct check before relying on this as a currently operating office.</t>
+          <t>Backed Unconventional AI, Physical Intelligence; ranked #2 in CNBC's 2026 list. | AUM figures found range wildly ($12B direct investments, $107.8B, $200B+) depending on whether Amazon stock/total net worth is conflated with actual family-office-managed direct-investment assets. No single figure could be confidently attributed as 'Bezos Expeditions AUM' specifically - left blank rather than pick a misleading number.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bezos Expeditions</t>
+          <t>Biltmore Family Office, LLC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Single-Family Office</t>
+          <t>Multi-Family Office</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Jeff Bezos</t>
+          <t>Chris Cecil</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Principal</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+          <t>Founder &amp; President</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>chris@biltmorefamilyoffice.com</t>
+        </is>
+      </c>
       <c r="F8" t="b">
         <v>0</v>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>+1 704-560-9288</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/chris-cecil-9701b818/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/biltmore-family-office-llc</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.bezosexpeditions.com</t>
+          <t>https://www.biltmorefamilyoffice.com</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Mercer Island</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>NC</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1320,30 +1340,34 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>$3.5B (per FinTrx)</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Founder-investor philosophy prioritizing transformative companies pursuing large market opportunities; willing to hold for very long time horizons. Favors direct founder relationships over intermediary fund managers.</t>
+          <t>Proprietary 'family balance sheet' framework integrating investments, wealth transfer/tax planning, family governance/education, and reporting. Goal: grow family assets over inflation, spending, taxes, liabilities, and generational expansion. Founding partners are fee-paying clients themselves, investing alongside the families they serve.</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Biotech, fintech, AI/robotics, space/aerospace, media, real estate, logistics, healthcare, education</t>
+          <t>Diversified multi-asset portfolios integrated with tax/estate planning</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Jeff Bezos's personal investment vehicle, based on Mercer Island, WA. Backs transformative companies across biotech, fintech, AI/robotics, space, media, real estate, logistics, healthcare, and education.</t>
+          <t>Founded 2008 by Chris Cecil, a great-grandson of George Vanderbilt; began serving outside clients in 2013.</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Backed Unconventional AI and Physical Intelligence; ranked #2 in CNBC's 2026 Family Office 15. Backed five AI startups in June 2026 per separate CNBC coverage.</t>
+          <t>Most recent 13F filing (2026-05-11) shows a position in Apple Inc. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="T8" t="b">
@@ -1351,37 +1375,37 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Backed Unconventional AI, Physical Intelligence; ranked #2 in CNBC's 2026 list.</t>
+          <t>Founded 2008 by Chris Cecil (great-grandson of George Vanderbilt) originally for Vanderbilt/Biltmore Estate wealth, but began serving outside clients in 2013 - now a 'collaborative family office group' for 'high-net-worth individuals, families, and their related entities'. Current state is multi-family, not single, despite single-family origin.</t>
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>press_named_sfo</t>
+          <t>own_website</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.cnbc.com/2026/02/12/inside-wealth-family-office-15.html</t>
+          <t>own_website: https://www.biltmorefamilyoffice.com/our-history/</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>Backed Unconventional AI, Physical Intelligence; ranked #2 in CNBC's 2026 list. | AUM figures found range wildly ($12B direct investments, $107.8B, $200B+) depending on whether Amazon stock/total net worth is conflated with actual family-office-managed direct-investment assets. No single figure could be confidently attributed as 'Bezos Expeditions AUM' specifically - left blank rather than pick a misleading number.</t>
+          <t>13F-HR filer, matched keyword 'family office'. Location: Charlotte, NC. | Single consistent source (firm bio page), domain-matched email - not deliverability-confirmed.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Biltmore Family Office, LLC</t>
+          <t>CVA Family Office, LLC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1391,50 +1415,38 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Chris Cecil</t>
+          <t>Matt Blackburn, Chris Younger, David Tolson, Dalyce Tinoco</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Founder &amp; President</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>chris@biltmorefamilyoffice.com</t>
-        </is>
-      </c>
+          <t>Co-Founders (Blackburn: Managing Partner)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="b">
         <v>0</v>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>+1 704-560-9288</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/chris-cecil-9701b818/</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/biltmore-family-office-llc</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/in/mattblackburnclassvi/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.biltmorefamilyoffice.com</t>
+          <t>https://classvifamilyoffice.com</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1442,34 +1454,30 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>$3.5B (per FinTrx)</t>
-        </is>
-      </c>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Proprietary 'family balance sheet' framework integrating investments, wealth transfer/tax planning, family governance/education, and reporting. Goal: grow family assets over inflation, spending, taxes, liabilities, and generational expansion. Founding partners are fee-paying clients themselves, investing alongside the families they serve.</t>
+          <t>Holistic, IPS-driven approach emphasizing strategic asset allocation, tax efficiency, and capital preservation for entrepreneurs/business owners, with particular focus on liquidity-event planning. Integrates investment banking and exit-planning services (via affiliated Class VI Partners) alongside wealth management.</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Diversified multi-asset portfolios integrated with tax/estate planning</t>
+          <t>Public and private markets, with investment-banking-adjacent liquidity-event planning for entrepreneurs</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Founded 2008 by Chris Cecil, a great-grandson of George Vanderbilt; began serving outside clients in 2013.</t>
+          <t>Founded September 2016, now operates as 'Class VI Family Office, LLC'. Focuses on HNW entrepreneurs and business owners.</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-05-11) shows a position in Apple Inc. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+          <t>Most recent 13F filing (2026-04-29) shows a position in Schwab Strategic Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="T9" t="b">
@@ -1477,7 +1485,7 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Founded 2008 by Chris Cecil (great-grandson of George Vanderbilt) originally for Vanderbilt/Biltmore Estate wealth, but began serving outside clients in 2013 - now a 'collaborative family office group' for 'high-net-worth individuals, families, and their related entities'. Current state is multi-family, not single, despite single-family origin.</t>
+          <t>Now operates as 'Class VI Family Office, LLC'. Founded 2016 by 4 unrelated co-founders (Blackburn, Younger, Tolson, Tinoco) as an RIA. Focuses on HNW entrepreneurs/business owners generally, not one family.</t>
         </is>
       </c>
       <c r="V9" t="n">
@@ -1485,12 +1493,12 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>own_website</t>
+          <t>multi_source_corroboration</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>own_website: https://www.biltmorefamilyoffice.com/our-history/</t>
+          <t>multi_source_corroboration: https://www.classvipartners.com/our-team/matt-blackburn/</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -1500,14 +1508,14 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>13F-HR filer, matched keyword 'family office'. Location: Charlotte, NC. | Single consistent source (firm bio page), domain-matched email - not deliverability-confirmed.</t>
+          <t>13F-HR filer, matched keyword 'family office'. Location: Denver, CO.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CVA Family Office, LLC</t>
+          <t>Callan Family Office, LLC</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1517,12 +1525,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Matt Blackburn, Chris Younger, David Tolson, Dalyce Tinoco</t>
+          <t>Jack Ginter</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Co-Founders (Blackburn: Managing Partner)</t>
+          <t>Founder &amp; CEO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -1532,23 +1540,27 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mattblackburnclassvi/</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>https://www.linkedin.com/in/jack-ginter-70276773/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/callan-family-office</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://classvifamilyoffice.com</t>
+          <t>https://callanfamilyoffice.com</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Radnor</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1556,30 +1568,34 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>$10.2B</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Holistic, IPS-driven approach emphasizing strategic asset allocation, tax efficiency, and capital preservation for entrepreneurs/business owners, with particular focus on liquidity-event planning. Integrates investment banking and exit-planning services (via affiliated Class VI Partners) alongside wealth management.</t>
+          <t>Core-satellite approach blending low-cost passive investment with high-conviction active management and private capital, optimized for after-tax/net-of-fee results. Leverages parent-adjacent Callan LLC's 45+ years of institutional research and ~2,000 annual manager due-diligence meetings.</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Public and private markets, with investment-banking-adjacent liquidity-event planning for entrepreneurs</t>
+          <t>Passive and active public market strategies plus private capital (core-satellite)</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Founded September 2016, now operates as 'Class VI Family Office, LLC'. Focuses on HNW entrepreneurs and business owners.</t>
+          <t>Founded 2022 by former Abbot Downing/Wells Fargo Private Bank executives; grew to 23 partners. 'Callan' is a licensed trademark from unrelated institutional consulting firm Callan LLC.</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-04-29) shows a position in Schwab Strategic Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+          <t>Most recent 13F filing (2026-05-13) shows a position in Nvidia Corporation. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="T10" t="b">
@@ -1587,20 +1603,20 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Now operates as 'Class VI Family Office, LLC'. Founded 2016 by 4 unrelated co-founders (Blackburn, Younger, Tolson, Tinoco) as an RIA. Focuses on HNW entrepreneurs/business owners generally, not one family.</t>
+          <t>Founded 2022 by Jack Ginter + 3 other named founding partners, grew to 23 partners who bought stakes. 'Callan' is a LICENSED TRADEMARK from an unrelated institutional consulting firm (Callan LLC), not a founder surname. $10.2B AUM, serves 'ultra-high net worth clients, family foundations, and endowments' - textbook example of 'family office' as marketing branding, not a real family name.</t>
         </is>
       </c>
       <c r="V10" t="n">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>multi_source_corroboration</t>
+          <t>press_named_sfo</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>multi_source_corroboration: https://www.classvipartners.com/our-team/matt-blackburn/</t>
+          <t>press_named_sfo: https://riabiz.com/a/2024/4/9/an-abbot-downing-breakaway-but-not-exactly-callan-family-office-hits-5-billion-of-aum-after-just-two-years-using-a-creative-callan-brand-deal-and-a-partnership-model</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -1610,14 +1626,14 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>13F-HR filer, matched keyword 'family office'. Location: Denver, CO.</t>
+          <t>13F-HR filer, matched keyword 'family office'. Location: Radnor, PA. | No email/phone found in public search results this pass.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Callan Family Office, LLC</t>
+          <t>Capitol Family Office, Inc.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1627,42 +1643,46 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Jack Ginter</t>
+          <t>Mark Nortman, Erica Nortman</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Founder &amp; CEO</t>
+          <t>Contacts/Principals</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="b">
         <v>0</v>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>503-897-0236</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jack-ginter-70276773/</t>
+          <t>https://www.linkedin.com/in/marknortman/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/callan-family-office</t>
+          <t>https://www.linkedin.com/company/capitol-family-office</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://callanfamilyoffice.com</t>
+          <t>https://capitolcfo.com</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Radnor</t>
+          <t>Beaverton</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1672,32 +1692,32 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>$10.2B</t>
+          <t>$136.5M</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Core-satellite approach blending low-cost passive investment with high-conviction active management and private capital, optimized for after-tax/net-of-fee results. Leverages parent-adjacent Callan LLC's 45+ years of institutional research and ~2,000 annual manager due-diligence meetings.</t>
+          <t>Discretionary asset management centered on pooled public equity vehicles (not bespoke single-stock portfolios). Not an active ESG investor; focused on long-term relationships with a select client group and intergenerational wealth preservation.</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Passive and active public market strategies plus private capital (core-satellite)</t>
+          <t>Pooled public equity vehicles</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Founded 2022 by former Abbot Downing/Wells Fargo Private Bank executives; grew to 23 partners. 'Callan' is a licensed trademark from unrelated institutional consulting firm Callan LLC.</t>
+          <t>Established 2011.</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-05-13) shows a position in Nvidia Corporation. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+          <t>Most recent 13F filing (2026-04-15) shows a position in Vanguard Index Fds. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="T11" t="b">
@@ -1705,20 +1725,20 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Founded 2022 by Jack Ginter + 3 other named founding partners, grew to 23 partners who bought stakes. 'Callan' is a LICENSED TRADEMARK from an unrelated institutional consulting firm (Callan LLC), not a founder surname. $10.2B AUM, serves 'ultra-high net worth clients, family foundations, and endowments' - textbook example of 'family office' as marketing branding, not a real family name.</t>
+          <t>Beaverton, OR, established 2011. Third-party source explicitly labels it a multi-family office. Contacts Mark and Erica Nortman.</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>press_named_sfo</t>
+          <t>third_party_directory</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://riabiz.com/a/2024/4/9/an-abbot-downing-breakaway-but-not-exactly-callan-family-office-hits-5-billion-of-aum-after-just-two-years-using-a-creative-callan-brand-deal-and-a-partnership-model</t>
+          <t>third_party_directory: https://www.retirementplanning.net/retirement-planners/oregon/beaverton/capitol-family-office-inc/2013080</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -1728,63 +1748,55 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>13F-HR filer, matched keyword 'family office'. Location: Radnor, PA. | No email/phone found in public search results this pass.</t>
+          <t>CAVEAT: multi-family classification rests only on a secondary aggregator label (e.g. Altss), not a primary quote from the firm itself. Not independently confirmed - same source class that was WRONG for Family Manage LLC (Altss said single-family, firm site said multi-family). Lower confidence than other MFO records in this file. Recommend a direct-site check before treating as equally solid. | 13F-HR filer, matched keyword 'family office'. Location: Beaverton, OR. | Very small team - only 2 employees, both investment professionals.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Capitol Family Office, Inc.</t>
+          <t>Cohen Private Ventures</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Multi-Family Office</t>
+          <t>Single-Family Office</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mark Nortman, Erica Nortman</t>
+          <t>Steven A. Cohen (Andrew B. Cohen: CIO/Co-Founder)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Contacts/Principals</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="b">
         <v>0</v>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>503-897-0236</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/marknortman/</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/capitol-family-office</t>
+          <t>https://www.linkedin.com/company/cohen-private-ventures</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://capitolcfo.com</t>
+          <t>https://www.cohenpv.com</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Beaverton</t>
+          <t>Stamford</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>OR</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1792,55 +1804,43 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>$136.5M</t>
-        </is>
-      </c>
+      <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Discretionary asset management centered on pooled public equity vehicles (not bespoke single-stock portfolios). Not an active ESG investor; focused on long-term relationships with a select client group and intergenerational wealth preservation.</t>
+          <t>Direct private equity, growth equity, and venture capital, plus structured securities, real estate, and credit - long-term capital deployment distinct from Point72's external-capital hedge fund strategies.</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Pooled public equity vehicles</t>
+          <t>Private equity, growth equity, venture capital, structured credit, real estate, special situations</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Established 2011.</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>Most recent 13F filing (2026-04-15) shows a position in Vanguard Index Fds. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
+          <t>Distinct from Point72 (Cohen's former hedge fund, converted 2016 to a multi-family office with outside capital). Invests in direct private equity, growth equity, VC, structured securities, real estate, credit.</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="b">
         <v>1</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Beaverton, OR, established 2011. Third-party source explicitly labels it a multi-family office. Contacts Mark and Erica Nortman.</t>
+          <t>Stamford, CT. Explicitly 'a single-family office of Steven A. Cohen', led by Andrew B. Cohen (CIO/Co-Founder). Invests in direct private equity, growth equity, VC, structured securities, real estate, credit. IMPORTANT DISTINCTION correctly kept separate: Cohen ALSO runs Point72 (the former hedge fund, converted 2016 to a multi-family office with outside capital) - Cohen Private Ventures is the distinct single-family vehicle, not Point72. Do not conflate the two if Point72 is ever separately discovered.</t>
         </is>
       </c>
       <c r="V12" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>third_party_directory</t>
+          <t>multi_source_corroboration</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>third_party_directory: https://www.retirementplanning.net/retirement-planners/oregon/beaverton/capitol-family-office-inc/2013080</t>
+          <t>multi_source_corroboration: https://familyofficehub.io/blog/the-cohen-family-office-cohen-private-ventures/</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -1850,55 +1850,59 @@
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>CAVEAT: multi-family classification rests only on a secondary aggregator label (e.g. Altss), not a primary quote from the firm itself. Not independently confirmed - same source class that was WRONG for Family Manage LLC (Altss said single-family, firm site said multi-family). Lower confidence than other MFO records in this file. Recommend a direct-site check before treating as equally solid. | 13F-HR filer, matched keyword 'family office'. Location: Beaverton, OR. | Very small team - only 2 employees, both investment professionals.</t>
+          <t>Press/database verified, not SEC-primary verified. | Multiple different 'Andrew Cohen' LinkedIn profiles surfaced (M. Cohen Capital, Greenoaks Capital, World Innovation Lab) - clearly different people sharing a common name. Could not confirm which, if any, is the Cohen Private Ventures CIO - left principal_linkedin blank rather than guess. | AUM not disclosed for Cohen Private Ventures itself. Point72 Asset Management ($45.7B AUM) is a separate, related entity (the converted multi-family-office successor to Cohen's original hedge fund) - its AUM is not CPV's own and is not used here.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cohen Private Ventures</t>
+          <t>Custos Family Office, LLC</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Single-Family Office</t>
+          <t>Multi-Family Office</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Steven A. Cohen (Andrew B. Cohen: CIO/Co-Founder)</t>
+          <t>Tony Lopiccolo, Mitchell Herr</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Founding Principal &amp; CIO (Lopiccolo)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="b">
         <v>0</v>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/cohen-private-ventures</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>303-536-5313 (Denver office)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/anthony-lopiccolo-cfa-b26aa519/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.cohenpv.com</t>
+          <t>https://custosfo.com</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Stamford</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1906,43 +1910,55 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>~$500-730M</t>
+        </is>
+      </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Direct private equity, growth equity, and venture capital, plus structured securities, real estate, and credit - long-term capital deployment distinct from Point72's external-capital hedge fund strategies.</t>
+          <t>Risk management across the client's entire balance sheet using client-specific profiles for asset allocation; implementation unconstrained by traditional asset classes (ETFs, institutional mutual funds, SMAs, private investments, hedging options). 100% partner-owned with no outside shareholders - explicitly framed as enabling full client-centricity.</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Private equity, growth equity, venture capital, structured credit, real estate, special situations</t>
+          <t>ETFs, institutional mutual funds, SMAs, private investments, hedging strategies</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Distinct from Point72 (Cohen's former hedge fund, converted 2016 to a multi-family office with outside capital). Invests in direct private equity, growth equity, VC, structured securities, real estate, credit.</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
+          <t>Founded 2018, partner-owned, fee-only. Team of 6 advisors.</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Most recent 13F filing (2026-02-17) shows a position in Ishares Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
       <c r="T13" t="b">
         <v>1</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Stamford, CT. Explicitly 'a single-family office of Steven A. Cohen', led by Andrew B. Cohen (CIO/Co-Founder). Invests in direct private equity, growth equity, VC, structured securities, real estate, credit. IMPORTANT DISTINCTION correctly kept separate: Cohen ALSO runs Point72 (the former hedge fund, converted 2016 to a multi-family office with outside capital) - Cohen Private Ventures is the distinct single-family vehicle, not Point72. Do not conflate the two if Point72 is ever separately discovered.</t>
+          <t>Austin TX, founded 2018, partner-owned (Tony Lopiccolo, Mitchell Herr), explicitly labeled multi-family office, serves 'affluent families' (plural), ~$500-730M AUM across 6 advisors.</t>
         </is>
       </c>
       <c r="V13" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>multi_source_corroboration</t>
+          <t>third_party_directory</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>multi_source_corroboration: https://familyofficehub.io/blog/the-cohen-family-office-cohen-private-ventures/</t>
+          <t>third_party_directory: https://custosfo.com/</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
@@ -1952,59 +1968,55 @@
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>Press/database verified, not SEC-primary verified. | Multiple different 'Andrew Cohen' LinkedIn profiles surfaced (M. Cohen Capital, Greenoaks Capital, World Innovation Lab) - clearly different people sharing a common name. Could not confirm which, if any, is the Cohen Private Ventures CIO - left principal_linkedin blank rather than guess. | AUM not disclosed for Cohen Private Ventures itself. Point72 Asset Management ($45.7B AUM) is a separate, related entity (the converted multi-family-office successor to Cohen's original hedge fund) - its AUM is not CPV's own and is not used here.</t>
+          <t>CAVEAT: multi-family classification rests only on a secondary aggregator label (e.g. Altss), not a primary quote from the firm itself. Not independently confirmed - same source class that was WRONG for Family Manage LLC (Altss said single-family, firm site said multi-family). Lower confidence than other MFO records in this file. Recommend a direct-site check before treating as equally solid. | 13F-HR filer, matched keyword 'family office'. Location: Littleton, CO. | No email/phone found in public search results this pass. | Email format pattern confirmed as [firstname]@custosfo.com (88% of firm emails), but no specific individual address confirmed - constructing tony@custosfo.com from the pattern alone would be a guess, not a verified fact, so left blank. Denver office phone: 303-536-5313.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Custos Family Office, LLC</t>
+          <t>DFO Management, LLC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Multi-Family Office</t>
+          <t>Single-Family Office</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tony Lopiccolo, Mitchell Herr</t>
+          <t>Michael Dell</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Founding Principal &amp; CIO (Lopiccolo)</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="b">
         <v>0</v>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>303-536-5313 (Denver office)</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/anthony-lopiccolo-cfa-b26aa519/</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/dfo-management</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://custosfo.com</t>
+          <t>https://www.dellfamilyoffice.com</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2012,34 +2024,30 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>~$500-730M</t>
-        </is>
-      </c>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Risk management across the client's entire balance sheet using client-specific profiles for asset allocation; implementation unconstrained by traditional asset classes (ETFs, institutional mutual funds, SMAs, private investments, hedging options). 100% partner-owned with no outside shareholders - explicitly framed as enabling full client-centricity.</t>
+          <t>Public equity positions via 13F filings include SafeHold Inc, Hayward Holdings Inc, and Townsquare Media Inc (as of the 2026-05-15 filing). Historically also active in private equity and real estate per press coverage.</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>ETFs, institutional mutual funds, SMAs, private investments, hedging strategies</t>
+          <t>Public equities, private equity, real estate (historical)</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Founded 2018, partner-owned, fee-only. Team of 6 advisors.</t>
+          <t>Founded 1998 by Michael Dell with John Phelan and Glenn Fuhrman as MSD Capital; restructured/rebranded as DFO Management, LLC in 2022. Historically invested across public equities, private equity, and real estate; the third-party-capital arm (MSD Partners) separately merged into BDT &amp; MSD Partners, a merchant bank, in 2023.</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-02-17) shows a position in Ishares Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+          <t>13F-reported public equity positions as of the most recent filing (2026-05-15): SafeHold Inc, Hayward Holdings Inc, Townsquare Media Inc. Position dollar values from this same filing pull were found implausible on cross-check and are not reported (see notes).</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="T14" t="b">
@@ -2047,30 +2055,30 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Austin TX, founded 2018, partner-owned (Tony Lopiccolo, Mitchell Herr), explicitly labeled multi-family office, serves 'affluent families' (plural), ~$500-730M AUM across 6 advisors.</t>
+          <t>Private investment firm for Michael Dell (Dell Technologies founder/CEO) and his family. Launched 1998 as MSD Capital, L.P.; rebranded DFO Management, LLC in 2022 following the 2023 merger of its affiliated third-party-capital arm (MSD Partners) with BDT &amp; Company. Confirmed via SEC EDGAR (CIK 1105497, active non-joint 13F-HR filings continuing under the legal name 'MSD Capital, L.P.' through 2026) and multiple independent sources (Wikipedia's dedicated 'DFO Management' article, family-office-advisory.com, the firm's own site dellfamilyoffice.com).</t>
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>third_party_directory</t>
+          <t>press_named_sfo, sec_13f_clean</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>third_party_directory: https://custosfo.com/</t>
+          <t>press_named_sfo: https://en.wikipedia.org/wiki/DFO_Management | sec_13f_clean: https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001105497&amp;type=13F-HR</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>CAVEAT: multi-family classification rests only on a secondary aggregator label (e.g. Altss), not a primary quote from the firm itself. Not independently confirmed - same source class that was WRONG for Family Manage LLC (Altss said single-family, firm site said multi-family). Lower confidence than other MFO records in this file. Recommend a direct-site check before treating as equally solid. | 13F-HR filer, matched keyword 'family office'. Location: Littleton, CO. | No email/phone found in public search results this pass. | Email format pattern confirmed as [firstname]@custosfo.com (88% of firm emails), but no specific individual address confirmed - constructing tony@custosfo.com from the pattern alone would be a guess, not a verified fact, so left blank. Denver office phone: 303-536-5313.</t>
+          <t>Rebranded from MSD Capital, L.P. to DFO Management, LLC in 2022; SEC 13F filings continue under the original registered legal name MSD Capital, L.P. (CIK 1105497) - both names verified as the same continuous entity via Wikipedia's dedicated article and the firm's own site (dellfamilyoffice.com), not just a name-similarity guess. CAVEAT: the SEC 13F bulk value pull for the 2026-05-15 filing listed SafeHold Inc at $78.24B - implausible, since Safehold's actual market cap is a small fraction of that. Same class of 13F value-parsing unreliability already documented in SYSTEM_DESIGN.md for other firms in this dataset. AUM and position dollar values are therefore left blank; only the confirmed identity of the holdings, not their claimed size, is reported. John Phelan is a long-standing co-founder/operating principal per press coverage; his exact current title following the 2022 rebrand and 2023 MSD Partners/BDT merger was not independently confirmed this session and is not asserted as principal_title.</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3503,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Hemendra Kothari Family Office</t>
+          <t>Henry Crown and Company</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3505,12 +3513,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Hemendra Kothari</t>
+          <t>Lester Crown, Bill Crown (A. Steven Crown: Executive Chairman)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Founder, Chairman &amp; Trustee</t>
+          <t>Directors (Henry Crown: Founder)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -3518,38 +3526,42 @@
         <v>0</v>
       </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/in/hemendra-kothari-302b3731a</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/henry-crown-&amp;-company</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Mumbai</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr"/>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Value investing prioritizing companies with strong fundamentals and experienced management; emphasis on diversification and long-term growth via fundamental analysis. Founded DSP Financial Consultants (1975), partnered with Merrill Lynch (1995), founded DSP Mutual Fund (2008, initially with BlackRock, later bought out BlackRock's stake).</t>
+          <t>Direct co-investments across private equity, real estate, infrastructure, and sports franchises, reflecting origins in industrial/manufacturing and real estate.</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Public equities (value investing); asset management (DSP Mutual Fund)</t>
+          <t>Direct co-investments, private equity, real estate, infrastructure, sports franchises</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>4th-generation stockbroking family; great-grandfather co-founded the Bombay Stock Exchange (1875). Founded DSP Financial Consultants, later DSP Merrill Lynch. Formerly President of the Bombay Stock Exchange.</t>
+          <t>Multi-generational: Henry -&gt; Lester -&gt; James Crown. Origins in Material Service Corp (coal/gravel/lime/sand), merged with General Dynamics.</t>
         </is>
       </c>
       <c r="R28" t="inlineStr"/>
@@ -3559,20 +3571,20 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Mumbai. Explicitly labeled 'single-family office' by SWFI and Altss ('Mumbai Single Family Office'). Manages multi-generational wealth, estate planning, philanthropy for the Kothari family.</t>
+          <t>Chicago. Direct explicit statement: 'Henry Crown and Company (HCC) is the family office for the Crown family.' Multi-generational (Henry -&gt; Lester -&gt; James Crown), currently directed by Lester and Bill Crown. Deploys capital via direct co-investments, PE, real estate, infrastructure, sports franchises. Multiply corroborated: BusinessWire, Altss ('Chicago Single Family Office'), Forbes family profile, multiple Wikipedia entries for family members.</t>
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.1</v>
+        <v>0.65</v>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>third_party_directory</t>
+          <t>press_named_sfo, multi_source_corroboration</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>third_party_directory: https://altss.com/profile/hemendra-kothari-family-office</t>
+          <t>press_named_sfo: https://www.businesswire.com/news/home/20250123832869/en/Henry-Crown-and-Company-Announces-New-Board-and-Leadership | multi_source_corroboration: https://altss.com/profile/cc-industries-inc-crown-family-office</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
@@ -3582,14 +3594,14 @@
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>CAVEAT: 'Kothari' is a common Indian surname with multiple distinct wealthy families with their own family offices (e.g. a separate 'Dr. Kulin Kothari Family Office' also exists, unrelated). The original NewsAPI article that surfaced 'Kothari Family Office' as a name did not clearly confirm which specific Kothari family it referred to - this record is my best-evidenced match, not a certain one. Foreign entity, press/database verified only. | Family group has evolved from fully family-run to professional day-to-day management; Aditi Kothari Desai (relation to Hemendra not fully confirmed) is Chairperson of DSP Asset Managers.</t>
+          <t>Press/database verified, not SEC-primary verified. | IMPORTANT: James Crown, listed elsewhere as a current active leader, died June 25, 2023. Current (2026) leadership of the firm was NOT confirmed in sources reviewed this session - this is an honest gap, not filled with a guess. Do not present James Crown as current active CEO without flagging this. | James S. Crown (former President/Chairman/CEO) died June 25, 2023 - current post-2023 day-to-day leadership not confirmed in sources reviewed. | IMPORTANT: James Crown, listed elsewhere as a current active leader, died June 25, 2023. Current (2026) leadership of the firm was NOT confirmed in sources reviewed this session - this is an honest gap, not filled with a guess. Do not present James Crown as current active CEO without flagging this. | Corporate LinkedIn confirmed via web search - official page, 1,100 followers, description matches known Chicago-based operations (real estate, public securities, investment funds).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Henry Crown and Company</t>
+          <t>Hillspire</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3599,12 +3611,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Lester Crown, Bill Crown (A. Steven Crown: Executive Chairman)</t>
+          <t>Eric Schmidt</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Directors (Henry Crown: Founder)</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -3615,18 +3627,18 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/henry-crown-&amp;-company</t>
+          <t>https://www.linkedin.com/company/hillspire-llc</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Menlo Park</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3634,60 +3646,72 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>$1-1.5B (range, per family-office database sources - not a precise disclosed figure)</t>
+        </is>
+      </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Direct co-investments across private equity, real estate, infrastructure, and sports franchises, reflecting origins in industrial/manufacturing and real estate.</t>
+          <t>Backs entrepreneurs leveraging breakthroughs in computing, AI, life sciences, and energy sustainability.</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Direct co-investments, private equity, real estate, infrastructure, sports franchises</t>
+          <t>AI, defense technology, biotechnology, climate technology</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Multi-generational: Henry -&gt; Lester -&gt; James Crown. Origins in Material Service Corp (coal/gravel/lime/sand), merged with General Dynamics.</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
+          <t>Family office of Eric and Wendy Schmidt (former Google CEO). Linked philanthropic entities confirmed via ProPublica: Schmidt Family Foundation (Chicago, IL) and Schmidt Ocean Institute (Palo Alto, CA).</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Ranked #1 in CNBC's inaugural Inside Wealth Family Office 15 (Feb 2026), 15 investments in 2025 mostly AI. Separately reported: 22 private AI company investments since 2019, combined funding rounds exceeding $5B, portfolio includes Anthropic and SandboxAQ.</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
       <c r="T29" t="b">
         <v>1</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Chicago. Direct explicit statement: 'Henry Crown and Company (HCC) is the family office for the Crown family.' Multi-generational (Henry -&gt; Lester -&gt; James Crown), currently directed by Lester and Bill Crown. Deploys capital via direct co-investments, PE, real estate, infrastructure, sports franchises. Multiply corroborated: BusinessWire, Altss ('Chicago Single Family Office'), Forbes family profile, multiple Wikipedia entries for family members.</t>
+          <t>Ranked #1 in CNBC's inaugural Inside Wealth Family Office 15 (2026), 15 investments in 2025, mostly AI.</t>
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.65</v>
+        <v>0.4</v>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>press_named_sfo, multi_source_corroboration</t>
+          <t>press_named_sfo</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.businesswire.com/news/home/20250123832869/en/Henry-Crown-and-Company-Announces-New-Board-and-Leadership | multi_source_corroboration: https://altss.com/profile/cc-industries-inc-crown-family-office</t>
+          <t>press_named_sfo: https://www.cnbc.com/2026/02/12/inside-wealth-family-office-15.html</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>Press/database verified, not SEC-primary verified. | IMPORTANT: James Crown, listed elsewhere as a current active leader, died June 25, 2023. Current (2026) leadership of the firm was NOT confirmed in sources reviewed this session - this is an honest gap, not filled with a guess. Do not present James Crown as current active CEO without flagging this. | James S. Crown (former President/Chairman/CEO) died June 25, 2023 - current post-2023 day-to-day leadership not confirmed in sources reviewed. | IMPORTANT: James Crown, listed elsewhere as a current active leader, died June 25, 2023. Current (2026) leadership of the firm was NOT confirmed in sources reviewed this session - this is an honest gap, not filled with a guess. Do not present James Crown as current active CEO without flagging this. | Corporate LinkedIn confirmed via web search - official page, 1,100 followers, description matches known Chicago-based operations (real estate, public securities, investment funds).</t>
+          <t>Ranked #1 in CNBC's inaugural Inside Wealth Family Office 15 (2026), 15 investments in 2025, mostly AI. | City/state (Reno, NV) is commonly cited for Hillspire but was NOT independently verified this session - treat as lower-confidence until confirmed. | CORRECTION: earlier city (Reno, NV) was explicitly flagged as unverified and is now confirmed wrong - corrected to Menlo Park, CA. Also: one source states Hillspire 'oversees capital for an additional California-based family' beyond the Schmidts - worth a closer look before assuming pure single-family exclusivity, though existing SFO qualification evidence (CNBC, ProPublica) remains independently strong.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Hillspire</t>
+          <t>Icahn Capital LP</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3697,7 +3721,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Eric Schmidt</t>
+          <t>Carl Icahn</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3713,18 +3737,22 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/hillspire-llc</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/icahn-capital-lp</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://carlicahn.com</t>
+        </is>
+      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Menlo Park</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3734,106 +3762,106 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>$1-1.5B (range, per family-office database sources - not a precise disclosed figure)</t>
+          <t>~$8.5B in disclosed 13F equity holdings (cash positions not publicly disclosed, so this understates total AUM)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Backs entrepreneurs leveraging breakthroughs in computing, AI, life sciences, and energy sustainability.</t>
+          <t>Classic activist model: acquire a significant stake in an undervalued/mismanaged public company, seek board representation via 13D filings, publicly advocate for change (asset sales, capital return, restructuring). Highly concentrated and idiosyncratic portfolio by design - influence over diversification. At 88, Icahn remains the primary decision-maker after five decades of activist investing.</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>AI, defense technology, biotechnology, climate technology</t>
+          <t>Public equities - concentrated activist positions, energy and restructuring plays</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Family office of Eric and Wendy Schmidt (former Google CEO). Linked philanthropic entities confirmed via ProPublica: Schmidt Family Foundation (Chicago, IL) and Schmidt Ocean Institute (Palo Alto, CA).</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>Ranked #1 in CNBC's inaugural Inside Wealth Family Office 15 (Feb 2026), 15 investments in 2025 mostly AI. Separately reported: 22 private AI company investments since 2019, combined funding rounds exceeding $5B, portfolio includes Anthropic and SandboxAQ.</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>2026-02-12</t>
-        </is>
-      </c>
+          <t>Distinct from Icahn Enterprises (IEP), Icahn's publicly-traded Nasdaq holding company with public shareholders - IEP is not a family office.</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
       <c r="T30" t="b">
         <v>1</v>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Ranked #1 in CNBC's inaugural Inside Wealth Family Office 15 (2026), 15 investments in 2025, mostly AI.</t>
+          <t>New York. 'A New York-based single family office that invests and manages all of Carl Icahn's assets' / 'manages the wealth of the Carl Icahn family.' IMPORTANT: this is DISTINCT from 'Icahn Enterprises' (IEP), Icahn's publicly-traded holding company on Nasdaq with public shareholders - that entity is explicitly NOT a family office (it's publicly traded) and must not be confused with or substituted for Icahn Capital LP.</t>
         </is>
       </c>
       <c r="V30" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>press_named_sfo</t>
+          <t>third_party_directory</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.cnbc.com/2026/02/12/inside-wealth-family-office-15.html</t>
+          <t>third_party_directory: https://www.preqin.com/data/profile/investor/icahn-capital/627067</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>Ranked #1 in CNBC's inaugural Inside Wealth Family Office 15 (2026), 15 investments in 2025, mostly AI. | City/state (Reno, NV) is commonly cited for Hillspire but was NOT independently verified this session - treat as lower-confidence until confirmed. | CORRECTION: earlier city (Reno, NV) was explicitly flagged as unverified and is now confirmed wrong - corrected to Menlo Park, CA. Also: one source states Hillspire 'oversees capital for an additional California-based family' beyond the Schmidts - worth a closer look before assuming pure single-family exclusivity, though existing SFO qualification evidence (CNBC, ProPublica) remains independently strong.</t>
+          <t>Press/database verified, not SEC-primary verified. | Corporate LinkedIn confirmed via web search - official page, address matches known White Plains, NY location. Low follower count (12) noted as a caveat, not treated as disqualifying since many private family offices deliberately keep minimal social presence.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Icahn Capital LP</t>
+          <t>Independent Family Office, LLC</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Single-Family Office</t>
+          <t>Multi-Family Office</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Carl Icahn</t>
+          <t>W. Michael Reickert</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="b">
         <v>0</v>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>518-452-8050</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/independent-family-office-llc</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/icahn-capital-lp</t>
+          <t>https://www.linkedin.com/company/independent-family-office-llc</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://carlicahn.com</t>
+          <t>https://ifollc.com</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Albany</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3848,32 +3876,40 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>~$8.5B in disclosed 13F equity holdings (cash positions not publicly disclosed, so this understates total AUM)</t>
+          <t>$618M discretionary (more precise figure found this pass)</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Classic activist model: acquire a significant stake in an undervalued/mismanaged public company, seek board representation via 13D filings, publicly advocate for change (asset sales, capital return, restructuring). Highly concentrated and idiosyncratic portfolio by design - influence over diversification. At 88, Icahn remains the primary decision-maker after five decades of activist investing.</t>
+          <t>Customized programs using fundamental and technical analysis; toolkit includes options/derivatives, short sales, margin borrowing, and hedge fund/PE allocations when appropriate. Primary focus is non-investment family office functions (estate planning support, day-to-day administration) alongside investment oversight.</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Public equities - concentrated activist positions, energy and restructuring plays</t>
+          <t>Options/derivatives, short sales, margin strategies, hedge funds, private equity</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>Distinct from Icahn Enterprises (IEP), Icahn's publicly-traded Nasdaq holding company with public shareholders - IEP is not a family office.</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
+          <t>Founded 2005 after Reickert led the family office practice at the Ayco Company.</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Most recent 13F filing (2026-05-15) shows a position in Ishares Gold Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
       <c r="T31" t="b">
         <v>1</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>New York. 'A New York-based single family office that invests and manages all of Carl Icahn's assets' / 'manages the wealth of the Carl Icahn family.' IMPORTANT: this is DISTINCT from 'Icahn Enterprises' (IEP), Icahn's publicly-traded holding company on Nasdaq with public shareholders - that entity is explicitly NOT a family office (it's publicly traded) and must not be confused with or substituted for Icahn Capital LP.</t>
+          <t>Albany NY, founded 2005 by W. Michael Reickert after leading the 'family office practice' at Ayco Company (a larger advisory firm) - an advisory-services career background, not a private family's own vehicle. Altss explicitly labels it 'Albany Multi Family Office'.</t>
         </is>
       </c>
       <c r="V31" t="n">
@@ -3886,7 +3922,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>third_party_directory: https://www.preqin.com/data/profile/investor/icahn-capital/627067</t>
+          <t>third_party_directory: https://ifollc.com/</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
@@ -3896,98 +3932,70 @@
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>Press/database verified, not SEC-primary verified. | Corporate LinkedIn confirmed via web search - official page, address matches known White Plains, NY location. Low follower count (12) noted as a caveat, not treated as disqualifying since many private family offices deliberately keep minimal social presence.</t>
+          <t>CAVEAT: multi-family classification rests only on a secondary aggregator label (e.g. Altss), not a primary quote from the firm itself. Not independently confirmed - same source class that was WRONG for Family Manage LLC (Altss said single-family, firm site said multi-family). Lower confidence than other MFO records in this file. Recommend a direct-site check before treating as equally solid. | 13F-HR filer, matched keyword 'family office'. Location: Albany, NY. | Phone is the firm main line. principal_linkedin here is the COMPANY page, not a personal profile - no personal profile found for Reickert.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Independent Family Office, LLC</t>
+          <t>Jaws Estates Capital</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Multi-Family Office</t>
+          <t>Single-Family Office</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>W. Michael Reickert</t>
+          <t>Barry Sternlicht</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>Founder &amp; Chief Investment Officer (also Chairman/CEO of Starwood Capital Group, ~$52B AUM)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="b">
         <v>0</v>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>518-452-8050</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/independent-family-office-llc</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/independent-family-office-llc</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://ifollc.com</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Albany</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>$618M discretionary (more precise figure found this pass)</t>
-        </is>
-      </c>
+          <t>https://www.jawsvc.com</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Customized programs using fundamental and technical analysis; toolkit includes options/derivatives, short sales, margin borrowing, and hedge fund/PE allocations when appropriate. Primary focus is non-investment family office functions (estate planning support, day-to-day administration) alongside investment oversight.</t>
+          <t>Long-duration mandate investing Sternlicht's own capital (no third-party funds raised) across real estate, venture capital, private equity, and public equities. Confirmed technology emphasis: AI/ML, Web3, enterprise software. ~22 investments made.</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Options/derivatives, short sales, margin strategies, hedge funds, private equity</t>
+          <t>Real estate, venture capital, private equity, public equities; AI/ML, Web3, enterprise software</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Founded 2005 after Reickert led the family office practice at the Ayco Company.</t>
+          <t>Linked philanthropic entities confirmed via ProPublica: The Barry S Sternlicht Foundation and Barry And Mimi Sternlicht Foundation (both Wilmington, DE), indicating spouse Mimi Sternlicht.</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-05-15) shows a position in Ishares Gold Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+          <t>Listed among most active family offices for 2025 dealmaking per CNBC's Inside Wealth Family Office 15.</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="T32" t="b">
@@ -3995,37 +4003,37 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Albany NY, founded 2005 by W. Michael Reickert after leading the 'family office practice' at Ayco Company (a larger advisory firm) - an advisory-services career background, not a private family's own vehicle. Altss explicitly labels it 'Albany Multi Family Office'.</t>
+          <t>Listed among most active family offices for 2025 dealmaking per CNBC.</t>
         </is>
       </c>
       <c r="V32" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>third_party_directory</t>
+          <t>press_named_sfo</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>third_party_directory: https://ifollc.com/</t>
+          <t>press_named_sfo: https://www.cnbc.com/2026/02/12/inside-wealth-family-office-15.html</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>CAVEAT: multi-family classification rests only on a secondary aggregator label (e.g. Altss), not a primary quote from the firm itself. Not independently confirmed - same source class that was WRONG for Family Manage LLC (Altss said single-family, firm site said multi-family). Lower confidence than other MFO records in this file. Recommend a direct-site check before treating as equally solid. | 13F-HR filer, matched keyword 'family office'. Location: Albany, NY. | Phone is the firm main line. principal_linkedin here is the COMPANY page, not a personal profile - no personal profile found for Reickert.</t>
+          <t>Listed among most active family offices for 2025 dealmaking per CNBC. | AUM not publicly disclosed for Jaws Estates Capital itself. Starwood Capital Group (~$120B AUM) is described as a PARALLEL vehicle, not a subsidiary - its AUM figure is not Jaws Estates Capital's own and is not used here.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jaws Estates Capital</t>
+          <t>Jones Family Office</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4035,12 +4043,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Barry Sternlicht</t>
+          <t>Paul Tudor Jones II</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Founder &amp; Chief Investment Officer (also Chairman/CEO of Starwood Capital Group, ~$52B AUM)</t>
+          <t>Founder (Tudor Investment Corporation)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -4050,76 +4058,76 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>https://www.jawsvc.com</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Greenwich</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Long-duration mandate investing Sternlicht's own capital (no third-party funds raised) across real estate, venture capital, private equity, and public equities. Confirmed technology emphasis: AI/ML, Web3, enterprise software. ~22 investments made.</t>
+          <t>Global macro investing across equities, fixed income, currencies, and commodities based on macroeconomic analysis and market timing. Allocates across commodities, hedge funds, private equity, real estate, and infrastructure; geographic reach spans North America, Africa, Europe, and Asia; stages from seed through middle market.</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Real estate, venture capital, private equity, public equities; AI/ML, Web3, enterprise software</t>
+          <t>Commodities, hedge funds, private equity, real estate, infrastructure</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>Linked philanthropic entities confirmed via ProPublica: The Barry S Sternlicht Foundation and Barry And Mimi Sternlicht Foundation (both Wilmington, DE), indicating spouse Mimi Sternlicht.</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>Listed among most active family offices for 2025 dealmaking per CNBC's Inside Wealth Family Office 15.</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>2026-02-12</t>
-        </is>
-      </c>
+          <t>Manages wealth through direct investments and partnerships across commodities, hedge funds, private equity, real estate, infrastructure. Distinct from Tudor Investment Corporation, his hedge fund (retains outside capital).</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
       <c r="T33" t="b">
         <v>1</v>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Listed among most active family offices for 2025 dealmaking per CNBC.</t>
+          <t>Greenwich, CT. 'The single-family office for Paul Tudor Jones, founder of Tudor Investments' - distinct from Tudor Investment Corporation (his hedge fund, which retains outside capital). Manages wealth through direct investments and partnerships across commodities, hedge funds, private equity, real estate, infrastructure. Multiply corroborated: Private Equity International, Altss ('Greenwich Single Family Office'), Buzzfile.</t>
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>press_named_sfo</t>
+          <t>multi_source_corroboration</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.cnbc.com/2026/02/12/inside-wealth-family-office-15.html</t>
+          <t>multi_source_corroboration: https://altss.com/profile/jones-family-office-paul-tudor-jones-ii-family-office</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>Listed among most active family offices for 2025 dealmaking per CNBC. | AUM not publicly disclosed for Jaws Estates Capital itself. Starwood Capital Group (~$120B AUM) is described as a PARALLEL vehicle, not a subsidiary - its AUM figure is not Jaws Estates Capital's own and is not used here.</t>
+          <t>Press/database verified, not SEC-primary verified. | IMPORTANT: jonesfamilyinvestment.com belongs to an unrelated 'Jones Family Investment Group' (Orange County, CA) - NOT Paul Tudor Jones's office (Greenwich, CT). Excluded from website field to avoid a wrong-entity error. No confirmed website found for the correct entity.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Jones Family Office</t>
+          <t>Kemnay Advisory Services</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4129,12 +4137,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Paul Tudor Jones II</t>
+          <t>Alan M. Parker</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Founder (Tudor Investment Corporation)</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -4143,16 +4151,20 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/kemnay-advisory-services-inc</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Greenwich</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4163,94 +4175,106 @@
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Global macro investing across equities, fixed income, currencies, and commodities based on macroeconomic analysis and market timing. Allocates across commodities, hedge funds, private equity, real estate, and infrastructure; geographic reach spans North America, Africa, Europe, and Asia; stages from seed through middle market.</t>
+          <t>Diversified across private equity, hedge funds, secondaries, real estate, and public equities, aimed at multigenerational capital preservation.</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Commodities, hedge funds, private equity, real estate, infrastructure</t>
+          <t>Private equity, hedge funds, secondaries, real estate, public equities</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>Manages wealth through direct investments and partnerships across commodities, hedge funds, private equity, real estate, infrastructure. Distinct from Tudor Investment Corporation, his hedge fund (retains outside capital).</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
+          <t>Formed 2012 by Alan M. Parker after the 1997 sale of a 20% stake in Duty Free Shoppers Group to LVMH. Directed by the Parker family from Geneva with operational ties to New York. Investment advisor support from PJT Park Hill since 2022.</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Increased Coinbase position ~44% in Q4 2025 per CNBC 13F coverage. NOTE: the raw 13F table total (~$622B) is NOT usable as an AUM figure - see SYSTEM_DESIGN.md for why.</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
       <c r="T34" t="b">
         <v>1</v>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Greenwich, CT. 'The single-family office for Paul Tudor Jones, founder of Tudor Investments' - distinct from Tudor Investment Corporation (his hedge fund, which retains outside capital). Manages wealth through direct investments and partnerships across commodities, hedge funds, private equity, real estate, infrastructure. Multiply corroborated: Private Equity International, Altss ('Greenwich Single Family Office'), Buzzfile.</t>
+          <t>Increased Coinbase position ~44% in Q4 2025 per CNBC 13F coverage.</t>
         </is>
       </c>
       <c r="V34" t="n">
-        <v>0.25</v>
+        <v>0.7</v>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>multi_source_corroboration</t>
+          <t>press_named_sfo, sec_13f_clean</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>multi_source_corroboration: https://altss.com/profile/jones-family-office-paul-tudor-jones-ii-family-office</t>
+          <t>press_named_sfo: https://www.cnbc.com/2026/02/26/billionaire-family-office-investments.html | sec_13f_clean: https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=1555283&amp;type=13F-HR</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>Press/database verified, not SEC-primary verified. | IMPORTANT: jonesfamilyinvestment.com belongs to an unrelated 'Jones Family Investment Group' (Orange County, CA) - NOT Paul Tudor Jones's office (Greenwich, CT). Excluded from website field to avoid a wrong-entity error. No confirmed website found for the correct entity.</t>
+          <t>Increased Coinbase position ~44% in Q4 2025 per CNBC 13F coverage. | Address refined: 45 Rockefeller Plaza, New York, NY 10020. NOTE: a LinkedIn profile for an 'Alan Parker' at 'Enterprise Marketing Blueprint LLC' surfaced in search but is explicitly a DIFFERENT unrelated person - not used, to avoid a wrong-person contact error. | A third-party aggregator figure ("$622,333,000") surfaced during AUM research - digits match the $622.3B 13F tableValueTotal already flagged in SYSTEM_DESIGN.md as unreliable/likely-not-representative of the Parker family's own AUM (unit-labeling ambiguity). Not adding a new AUM figure to avoid restating the same unreliable number under a different label.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Kemnay Advisory Services</t>
+          <t>Kopp Family Office, LLC</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Single-Family Office</t>
+          <t>Multi-Family Office</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Alan M. Parker</t>
+          <t>LeRoy 'Lee' C. Kopp (d. 2020)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Principal</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr"/>
+          <t>Founder (Lindsey Lang: current President)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>foundation@koppfam.com</t>
+        </is>
+      </c>
       <c r="F35" t="b">
         <v>0</v>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>952-841-0438</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/kemnay-advisory-services-inc</t>
-        </is>
-      </c>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Bloomington</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4261,27 +4285,27 @@
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Diversified across private equity, hedge funds, secondaries, real estate, and public equities, aimed at multigenerational capital preservation.</t>
+          <t>Institutional approach focused on directly-managed public equities and ETFs plus opportunistic allocations (not external fund commitments); consolidated reporting, tax planning, governance support. Activity confined to North America.</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Private equity, hedge funds, secondaries, real estate, public equities</t>
+          <t>Public equities and ETFs (directly managed)</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Formed 2012 by Alan M. Parker after the 1997 sale of a 20% stake in Duty Free Shoppers Group to LVMH. Directed by the Parker family from Geneva with operational ties to New York. Investment advisor support from PJT Park Hill since 2022.</t>
+          <t>Established 2016 after Kopp's decades running Kopp Investment Advisors. Related Kopp Family Foundation is a real, active philanthropic entity.</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Increased Coinbase position ~44% in Q4 2025 per CNBC 13F coverage. NOTE: the raw 13F table total (~$622B) is NOT usable as an AUM figure - see SYSTEM_DESIGN.md for why.</t>
+          <t>Most recent 13F filing (2026-07-09) shows a position in Ishares Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="T35" t="b">
@@ -4289,37 +4313,37 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>Increased Coinbase position ~44% in Q4 2025 per CNBC 13F coverage.</t>
+          <t>Bloomington MN, established 2016 by LeRoy 'Lee' Kopp after decades running Kopp Investment Advisors (a prior general RIA). Altss labels it 'Bloomington Multi Family Office'; no contradicting evidence found. Lee Kopp died 2020, related Kopp Family Foundation is a real philanthropic entity, current president Lindsey Lang.</t>
         </is>
       </c>
       <c r="V35" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>press_named_sfo, sec_13f_clean</t>
+          <t>third_party_directory</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.cnbc.com/2026/02/26/billionaire-family-office-investments.html | sec_13f_clean: https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=1555283&amp;type=13F-HR</t>
+          <t>third_party_directory: https://altss.com/profile/kopp-family-office-llc</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>Increased Coinbase position ~44% in Q4 2025 per CNBC 13F coverage. | Address refined: 45 Rockefeller Plaza, New York, NY 10020. NOTE: a LinkedIn profile for an 'Alan Parker' at 'Enterprise Marketing Blueprint LLC' surfaced in search but is explicitly a DIFFERENT unrelated person - not used, to avoid a wrong-person contact error. | A third-party aggregator figure ("$622,333,000") surfaced during AUM research - digits match the $622.3B 13F tableValueTotal already flagged in SYSTEM_DESIGN.md as unreliable/likely-not-representative of the Parker family's own AUM (unit-labeling ambiguity). Not adding a new AUM figure to avoid restating the same unreliable number under a different label.</t>
+          <t>CAVEAT: multi-family classification rests only on a secondary aggregator label (e.g. Altss), not a primary quote from the firm itself. Not independently confirmed - same source class that was WRONG for Family Manage LLC (Altss said single-family, firm site said multi-family). Lower confidence than other MFO records in this file. Recommend a direct-site check before treating as equally solid. | 13F-HR filer, matched keyword 'family office'. Location: Bloomington, MN. | IMPORTANT CAVEAT: this phone/email is for the Kopp Family FOUNDATION (a separate 501c3 philanthropic entity), not confirmed as the Family Office's own line - Lindsey Lang is President of both and they share an address (8500 Normandale Lake Blvd Suite 475, Bloomington MN), but they are legally distinct entities. Included as the best available proxy contact, not a confirmed direct line. | Only the related Kopp Family FOUNDATION has a public website (koppfamilyfoundation.org) - a separate 501c3 entity, not used here to avoid misattributing it as the Family Office's own site. No dedicated Family Office website found.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Kopp Family Office, LLC</t>
+          <t>LBJ Family Wealth Advisors, Ltd.</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4329,38 +4353,38 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LeRoy 'Lee' C. Kopp (d. 2020)</t>
+          <t>Luci Baines Johnson</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Founder (Lindsey Lang: current President)</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>foundation@koppfam.com</t>
-        </is>
-      </c>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
       <c r="F36" t="b">
         <v>0</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>952-841-0438</t>
+          <t>512-457-5000 (firm main line)</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://lbjadvisors.com</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Bloomington</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4371,27 +4395,27 @@
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Institutional approach focused on directly-managed public equities and ETFs plus opportunistic allocations (not external fund commitments); consolidated reporting, tax planning, governance support. Activity confined to North America.</t>
+          <t>Holistic stewardship integrating investment strategy with family values/long-term planning. Relies on index ETFs/mutual funds and other money managers rather than individual securities for the core portfolio; may add PE/real estate/hard-asset limited partnerships for volatility reduction and inflation protection. Seeks low management fees.</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Public equities and ETFs (directly managed)</t>
+          <t>Index ETFs/mutual funds; selective private equity, real estate, hard assets</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Established 2016 after Kopp's decades running Kopp Investment Advisors. Related Kopp Family Foundation is a real, active philanthropic entity.</t>
+          <t>Founded 2003 by Luci Baines Johnson, daughter of President Lyndon B. Johnson and Lady Bird Johnson.</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-07-09) shows a position in Ishares Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+          <t>Most recent 13F filing (2026-07-14) top holding: Ishares Tr Rus 1000 Grw Etf, $45,912k.</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="T36" t="b">
@@ -4399,20 +4423,20 @@
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>Bloomington MN, established 2016 by LeRoy 'Lee' Kopp after decades running Kopp Investment Advisors (a prior general RIA). Altss labels it 'Bloomington Multi Family Office'; no contradicting evidence found. Lee Kopp died 2020, related Kopp Family Foundation is a real philanthropic entity, current president Lindsey Lang.</t>
+          <t>Austin TX, founded 2003 by Luci Baines Johnson (daughter of President Lyndon B. Johnson). CHECKED FIRM'S OWN SITE before assuming single-family from the famous name: explicitly states 'multi-generational, family-owned, family wealth management firm serving clients' (plural) and 'family-to-family not business-to-consumer' - serves external client families, not just the Johnson family. Notable enrichment detail regardless of type.</t>
         </is>
       </c>
       <c r="V36" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>third_party_directory</t>
+          <t>own_website</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>third_party_directory: https://altss.com/profile/kopp-family-office-llc</t>
+          <t>own_website: https://lbjadvisors.com/about/</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
@@ -4422,86 +4446,82 @@
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>CAVEAT: multi-family classification rests only on a secondary aggregator label (e.g. Altss), not a primary quote from the firm itself. Not independently confirmed - same source class that was WRONG for Family Manage LLC (Altss said single-family, firm site said multi-family). Lower confidence than other MFO records in this file. Recommend a direct-site check before treating as equally solid. | 13F-HR filer, matched keyword 'family office'. Location: Bloomington, MN. | IMPORTANT CAVEAT: this phone/email is for the Kopp Family FOUNDATION (a separate 501c3 philanthropic entity), not confirmed as the Family Office's own line - Lindsey Lang is President of both and they share an address (8500 Normandale Lake Blvd Suite 475, Bloomington MN), but they are legally distinct entities. Included as the best available proxy contact, not a confirmed direct line. | Only the related Kopp Family FOUNDATION has a public website (koppfamilyfoundation.org) - a separate 501c3 entity, not used here to avoid misattributing it as the Family Office's own site. No dedicated Family Office website found.</t>
+          <t>13F-HR filer, matched keyword 'family wealth'. Location: Austin, TX. | Full address: 3800 North Lamar, Suite 200, Austin, TX 78756. No phone/email found in public results.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>LBJ Family Wealth Advisors, Ltd.</t>
+          <t>Latsco Family Office</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Multi-Family Office</t>
+          <t>Single-Family Office</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Luci Baines Johnson</t>
+          <t>Marianna Latsis</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="b">
         <v>0</v>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>512-457-5000 (firm main line)</t>
-        </is>
-      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>https://lbjadvisors.com</t>
-        </is>
-      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://gr.linkedin.com/company/latsco-family-office</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Austin</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
+          <t>Athens</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr"/>
+          <t>Greece</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Latsis family net worth ~$2.2B (Forbes 2024) - not a precise firm AUM figure</t>
+        </is>
+      </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Holistic stewardship integrating investment strategy with family values/long-term planning. Relies on index ETFs/mutual funds and other money managers rather than individual securities for the core portfolio; may add PE/real estate/hard-asset limited partnerships for volatility reduction and inflation protection. Seeks low management fees.</t>
+          <t>Direct strategic investments and joint ventures (e.g. with EOS Capital Partners, Motor Oil) leveraging the family's shipping/energy heritage, expanding into infrastructure, real estate, fintech, and broader Greek-economy opportunities.</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Index ETFs/mutual funds; selective private equity, real estate, hard assets</t>
+          <t>Direct investments, private equity, real assets</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>Founded 2003 by Luci Baines Johnson, daughter of President Lyndon B. Johnson and Lady Bird Johnson.</t>
+          <t>Founded 2020, manages the Latsis family's shipping/energy fortune.</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-07-14) top holding: Ishares Tr Rus 1000 Grw Etf, $45,912k.</t>
+          <t>Joint 30% acquisition of Nova ICT with EOS Capital Partners (with Motor Oil); participation in Phaistos Investment Fund.</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="T37" t="b">
@@ -4509,20 +4529,20 @@
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>Austin TX, founded 2003 by Luci Baines Johnson (daughter of President Lyndon B. Johnson). CHECKED FIRM'S OWN SITE before assuming single-family from the famous name: explicitly states 'multi-generational, family-owned, family wealth management firm serving clients' (plural) and 'family-to-family not business-to-consumer' - serves external client families, not just the Johnson family. Notable enrichment detail regardless of type.</t>
+          <t>Athens, Greece. Founded 2020, manages the private wealth of the Latsis family (shipping/energy fortune). Explicitly labeled 'Athens Single Family Office' by Altss. Recent verified activity: joint 30% acquisition of Nova ICT with EOS Capital Partners (July 2026), participation in Phaistos Investment Fund.</t>
         </is>
       </c>
       <c r="V37" t="n">
-        <v>0.25</v>
+        <v>0.65</v>
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>own_website</t>
+          <t>press_named_sfo, multi_source_corroboration</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>own_website: https://lbjadvisors.com/about/</t>
+          <t>press_named_sfo: https://en.protothema.gr/2026/07/21/latsco-family-office-and-eos-capital-acquire-30-stake-in-nova-ict-in-partnership-with-motor-oil/ | multi_source_corroboration: https://altss.com/profile/latsco-family-office</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
@@ -4532,14 +4552,14 @@
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>13F-HR filer, matched keyword 'family wealth'. Location: Austin, TX. | Full address: 3800 North Lamar, Suite 200, Austin, TX 78756. No phone/email found in public results.</t>
+          <t>Foreign entity (Greece) - press/database verified, not SEC-primary verified. | Offices in Athens, Geneva, and London. In 2019 Marianna Latsis and siblings formally divided the broader family holdings; she took the helm of the shipping interests under Latsco specifically. | Corporate LinkedIn confirmed via web search - official page, 1,375 followers, matches known Athens headquarters and Latsis family ownership.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Latsco Family Office</t>
+          <t>Maelstrom</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4549,12 +4569,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Marianna Latsis</t>
+          <t>Arthur Hayes</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Founder / CIO (BitMEX co-founder)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -4565,49 +4585,41 @@
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://gr.linkedin.com/company/latsco-family-office</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>Athens</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/maelstromfund</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://maelstrom.fund</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>Greece</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>Latsis family net worth ~$2.2B (Forbes 2024) - not a precise firm AUM figure</t>
-        </is>
-      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Direct strategic investments and joint ventures (e.g. with EOS Capital Partners, Motor Oil) leveraging the family's shipping/energy heritage, expanding into infrastructure, real estate, fintech, and broader Greek-economy opportunities.</t>
+          <t>Early-stage crypto/decentralization infrastructure investing with a long-term, patient mandate; expanding into private-equity-style acquisitions of established mid-sized crypto-ecosystem businesses.</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>Direct investments, private equity, real assets</t>
+          <t>Crypto infrastructure, early-stage decentralization technology</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Founded 2020, manages the Latsis family's shipping/energy fortune.</t>
+          <t>Funded solely by Hayes, no outside LPs. Akshat Vaidya serves as investment head.</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Joint 30% acquisition of Nova ICT with EOS Capital Partners (with Motor Oil); participation in Phaistos Investment Fund.</t>
+          <t>Raising Maelstrom Equity Fund I, targeting $250M for 4-6 crypto-infrastructure acquisitions ($40-75M per deal).</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2025-10-17</t>
         </is>
       </c>
       <c r="T38" t="b">
@@ -4615,20 +4627,20 @@
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Athens, Greece. Founded 2020, manages the private wealth of the Latsis family (shipping/energy fortune). Explicitly labeled 'Athens Single Family Office' by Altss. Recent verified activity: joint 30% acquisition of Nova ICT with EOS Capital Partners (July 2026), participation in Phaistos Investment Fund.</t>
+          <t>Explicitly funded solely by Hayes himself with no outside LPs (limited partners) - directly confirms single-individual capital structure, not a pooled multi-investor fund. Bloomberg headline itself: 'Arthur Hayes' Family Office Seeks $250 Million for Buyout Fund'. Real recent activity: raising Maelstrom Equity Fund I ($250M target, $40-75M per deal, crypto-infrastructure acquisitions).</t>
         </is>
       </c>
       <c r="V38" t="n">
-        <v>0.65</v>
+        <v>0.4</v>
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>press_named_sfo, multi_source_corroboration</t>
+          <t>press_named_sfo</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://en.protothema.gr/2026/07/21/latsco-family-office-and-eos-capital-acquire-30-stake-in-nova-ict-in-partnership-with-motor-oil/ | multi_source_corroboration: https://altss.com/profile/latsco-family-office</t>
+          <t>press_named_sfo: https://www.bloomberg.com/news/articles/2025-10-17/arthur-hayes-family-office-seeks-250-million-for-buyout-fund</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
@@ -4638,14 +4650,14 @@
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>Foreign entity (Greece) - press/database verified, not SEC-primary verified. | Offices in Athens, Geneva, and London. In 2019 Marianna Latsis and siblings formally divided the broader family holdings; she took the helm of the shipping interests under Latsco specifically. | Corporate LinkedIn confirmed via web search - official page, 1,375 followers, matches known Athens headquarters and Latsis family ownership.</t>
+          <t>Press-verified (Bloomberg + own site), not SEC-primary verified. | Corporate LinkedIn confirmed via web search - official active page, corroborated by Arthur Hayes' own LinkedIn post referencing 'my family office Maelstrom' and the firm's own website (maelstrom.fund).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Maelstrom</t>
+          <t>Mousse Partners</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4655,12 +4667,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Arthur Hayes</t>
+          <t>Charles Heilbronn (founder; half-brother to owners Alain and Gerard Wertheimer)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Founder / CIO (BitMEX co-founder)</t>
+          <t>Founder (1991)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -4668,65 +4680,53 @@
         <v>0</v>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/maelstromfund</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>https://maelstrom.fund</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/charles-heilbronn-27984515b/</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Early-stage crypto/decentralization infrastructure investing with a long-term, patient mandate; expanding into private-equity-style acquisitions of established mid-sized crypto-ecosystem businesses.</t>
+          <t>Deep focus on the consumer sector - DTC brands, e-commerce, luxury goods, lifestyle companies, and consumer-experience technology - leveraging the Wertheimer family's brand-building and luxury-retail expertise. Long-term strategy across public/private markets, alternative investments, and collaborative partnerships with external managers.</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Crypto infrastructure, early-stage decentralization technology</t>
+          <t>Consumer/DTC brands, e-commerce, luxury goods, lifestyle, consumer technology</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>Funded solely by Hayes, no outside LPs. Akshat Vaidya serves as investment head.</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>Raising Maelstrom Equity Fund I, targeting $250M for 4-6 crypto-infrastructure acquisitions ($40-75M per deal).</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>2025-10-17</t>
-        </is>
-      </c>
+          <t>Invests across public/private equity, VC, credit, real assets. Offices in New York, Beijing, Hong Kong. Heilbronn holds board seats at Coty Inc. and Ulta Beauty representing family interests.</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
       <c r="T39" t="b">
         <v>1</v>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>Explicitly funded solely by Hayes himself with no outside LPs (limited partners) - directly confirms single-individual capital structure, not a pooled multi-investor fund. Bloomberg headline itself: 'Arthur Hayes' Family Office Seeks $250 Million for Buyout Fund'. Real recent activity: raising Maelstrom Equity Fund I ($250M target, $40-75M per deal, crypto-infrastructure acquisitions).</t>
+          <t>'Serves as a family office to manage the wealth of Alain and Gerard Wertheimer' (brothers, same lineage). Invests across public/private equity, VC, credit, real assets; offices in NY, Beijing, Hong Kong. PARTIAL US corroboration found: 'Mousseluxe Sarl' (CIK 1638286) and Charles Heilbronn (a known Wertheimer family representative) appear in real SEC insider filings (Forms 3/4) tied to Coty Inc. and Ulta Beauty board seats - confirms US market presence even though Mousse Partners itself isn't a direct 13F/ADV filer under that name.</t>
         </is>
       </c>
       <c r="V39" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>press_named_sfo</t>
+          <t>third_party_directory</t>
         </is>
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.bloomberg.com/news/articles/2025-10-17/arthur-hayes-family-office-seeks-250-million-for-buyout-fund</t>
+          <t>third_party_directory: https://en.wikipedia.org/wiki/Mousse_Partners</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
@@ -4736,83 +4736,119 @@
       </c>
       <c r="Z39" t="inlineStr">
         <is>
-          <t>Press-verified (Bloomberg + own site), not SEC-primary verified. | Corporate LinkedIn confirmed via web search - official active page, corroborated by Arthur Hayes' own LinkedIn post referencing 'my family office Maelstrom' and the firm's own website (maelstrom.fund).</t>
+          <t>Primarily press/Wikipedia-verified with partial SEC-adjacent corroboration (affiliated entity/individual insider filings), not a direct primary-source filing for Mousse Partners itself. | CORRECTION to earlier note: Heilbronn is not just a family representative - he is the firm's FOUNDER (1991) and the Wertheimer brothers' half-brother.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mousse Partners</t>
+          <t>Pathstone Family Office, LLC</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Single-Family Office</t>
+          <t>Multi-Family Office</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Charles Heilbronn (founder; half-brother to owners Alain and Gerard Wertheimer)</t>
+          <t>Steve Braverman, Allan Zachariah (Matthew Fleissig: current CEO)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Founder (1991)</t>
+          <t>Co-Founders</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="b">
         <v>0</v>
       </c>
-      <c r="G40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>201-944-7284 (firm main line)</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/charles-heilbronn-27984515b/</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
+          <t>https://www.linkedin.com/in/fleissig/</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/pathstone-family-office</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://pathstone.com</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Fort Lee</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>$125B standalone + $62B affiliate firms = ~$187B combined (as of Dec 31, 2025, post Hall Capital merger)</t>
+        </is>
+      </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Deep focus on the consumer sector - DTC brands, e-commerce, luxury goods, lifestyle companies, and consumer-experience technology - leveraging the Wertheimer family's brand-building and luxury-retail expertise. Long-term strategy across public/private markets, alternative investments, and collaborative partnerships with external managers.</t>
+          <t>Open-architecture, customized implementation via a global manager network. Active alternatives program (PE, VC, real estate, hedge funds) with rigorous quantitative/qualitative manager due diligence. Considers the family's total wealth picture - concentrated stock, real estate, business interests, philanthropy.</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Consumer/DTC brands, e-commerce, luxury goods, lifestyle, consumer technology</t>
+          <t>Private equity, venture capital, real estate, hedge funds (active alternatives program)</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>Invests across public/private equity, VC, credit, real assets. Offices in New York, Beijing, Hong Kong. Heilbronn holds board seats at Coty Inc. and Ulta Beauty representing family interests.</t>
-        </is>
-      </c>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
+          <t>Founded 2010 by former Harris myCFO managing directors. Also operates in Atlanta and Naples, FL.</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Most recent 13F filing (2023-11-08) shows a position in Spdr S&amp;P 500 Etf Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>2023-11-08</t>
+        </is>
+      </c>
       <c r="T40" t="b">
         <v>1</v>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>'Serves as a family office to manage the wealth of Alain and Gerard Wertheimer' (brothers, same lineage). Invests across public/private equity, VC, credit, real assets; offices in NY, Beijing, Hong Kong. PARTIAL US corroboration found: 'Mousseluxe Sarl' (CIK 1638286) and Charles Heilbronn (a known Wertheimer family representative) appear in real SEC insider filings (Forms 3/4) tied to Coty Inc. and Ulta Beauty board seats - confirms US market presence even though Mousse Partners itself isn't a direct 13F/ADV filer under that name.</t>
+          <t>Fort Lee NJ, founded 2010 by Steve Braverman and Allan Zachariah (unrelated ex-Harris myCFO executives). Explicitly 'partner-owned multi-family office' serving 'ultra-high net worth families, single family offices, foundations, and endowments'.</t>
         </is>
       </c>
       <c r="V40" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>third_party_directory</t>
+          <t>press_named_sfo</t>
         </is>
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>third_party_directory: https://en.wikipedia.org/wiki/Mousse_Partners</t>
+          <t>press_named_sfo: https://www.prnewswire.com/news-releases/pathstone-family-office-launches-independent-family-and-employee-owned-multi-family-office-95319759.html</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
@@ -4822,98 +4858,70 @@
       </c>
       <c r="Z40" t="inlineStr">
         <is>
-          <t>Primarily press/Wikipedia-verified with partial SEC-adjacent corroboration (affiliated entity/individual insider filings), not a direct primary-source filing for Mousse Partners itself. | CORRECTION to earlier note: Heilbronn is not just a family representative - he is the firm's FOUNDER (1991) and the Wertheimer brothers' half-brother.</t>
+          <t>13F-HR filer, matched keyword 'family office'. Location: Englewood, NJ. | Confirmed Matthew Fleissig is a CO-FOUNDER and current CEO, not just later-hired CEO - refines earlier note. No email/phone found.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Pathstone Family Office, LLC</t>
+          <t>Pontegadea Inversiones</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Multi-Family Office</t>
+          <t>Single-Family Office</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Steve Braverman, Allan Zachariah (Matthew Fleissig: current CEO)</t>
+          <t>Amancio Ortega</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Co-Founders</t>
+          <t>Founder (Zara/Inditex)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="b">
         <v>0</v>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>201-944-7284 (firm main line)</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/fleissig/</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/pathstone-family-office</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>https://pathstone.com</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Fort Lee</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>NJ</t>
-        </is>
-      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>$125B standalone + $62B affiliate firms = ~$187B combined (as of Dec 31, 2025, post Hall Capital merger)</t>
-        </is>
-      </c>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Open-architecture, customized implementation via a global manager network. Active alternatives program (PE, VC, real estate, hedge funds) with rigorous quantitative/qualitative manager due diligence. Considers the family's total wealth picture - concentrated stock, real estate, business interests, philanthropy.</t>
+          <t>All-cash acquisitions (no leverage) of premium commercial real estate, held in perpetuity for long-term cash flow rather than a 5-10 year exit horizon. Started 2001 using Inditex IPO proceeds.</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>Private equity, venture capital, real estate, hedge funds (active alternatives program)</t>
+          <t>Premium commercial real estate in major global capitals (London, New York, Miami, Toronto, Madrid, Paris)</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>Founded 2010 by former Harris myCFO managing directors. Also operates in Atlanta and Naples, FL.</t>
+          <t>De facto family office of Amancio Ortega; one of the largest single-family offices in Europe by assets. Net worth context ~$130B.</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2023-11-08) shows a position in Spdr S&amp;P 500 Etf Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+          <t>2025: $283M Barcelona office building (from Blackstone); 49% stake in UK's PD Ports (from Brookfield); $780M Vancouver building (from QuadReal).</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>2023-11-08</t>
+          <t>2025-11-24</t>
         </is>
       </c>
       <c r="T41" t="b">
@@ -4921,7 +4929,7 @@
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>Fort Lee NJ, founded 2010 by Steve Braverman and Allan Zachariah (unrelated ex-Harris myCFO executives). Explicitly 'partner-owned multi-family office' serving 'ultra-high net worth families, single family offices, foundations, and endowments'.</t>
+          <t>Spain-based. Described as 'the primary investment vehicle and de facto family office of Amancio Ortega... one of the largest single family offices in Europe by assets'. Very well documented, active 2025 dealflow: $283M Barcelona office building (from Blackstone), 49% stake in UK's PD Ports (from Brookfield), $780M Vancouver building (from QuadReal). Net worth context ~$130B.</t>
         </is>
       </c>
       <c r="V41" t="n">
@@ -4934,7 +4942,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.prnewswire.com/news-releases/pathstone-family-office-launches-independent-family-and-employee-owned-multi-family-office-95319759.html</t>
+          <t>press_named_sfo: https://www.caproasia.com/2026/04/26/spain-fashion-zara-founder-billionaire-amancio-ortega-age-90-with-130-billion-fortune-family-office-property-group-pontegadea-bought-more-than-1-5-billion-properties-in-north-america-europe/</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -4944,14 +4952,14 @@
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>13F-HR filer, matched keyword 'family office'. Location: Englewood, NJ. | Confirmed Matthew Fleissig is a CO-FOUNDER and current CEO, not just later-hired CEO - refines earlier note. No email/phone found.</t>
+          <t>Foreign entity, same caveat as Valhalla Ventures - press-verified only, no US SEC/ProPublica cross-check possible.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Pontegadea Inversiones</t>
+          <t>Soros Fund Management</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4961,12 +4969,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Amancio Ortega</t>
+          <t>George Soros</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Founder (Zara/Inditex)</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -4975,47 +4983,63 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/soros-fund-management</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://sorosfundmgmt.com</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr"/>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>~$28B net assets</t>
+        </is>
+      </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>All-cash acquisitions (no leverage) of premium commercial real estate, held in perpetuity for long-term cash flow rather than a 5-10 year exit horizon. Started 2001 using Inditex IPO proceeds.</t>
+          <t>Reflexivity-theory-informed: investor biases and market fundamentals form feedback loops affecting prices. Unconstrained global mandate across equities, credit, fixed income, macro, and private equity; takes large concentrated positions when conviction is high. Distinctively, the firm's stated primary mandate is to serve as the permanent capital base funding the Open Society Foundations.</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Premium commercial real estate in major global capitals (London, New York, Miami, Toronto, Madrid, Paris)</t>
+          <t>Equities, credit, fixed income, macro, private equity - technology and industrial exposure</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>De facto family office of Amancio Ortega; one of the largest single-family offices in Europe by assets. Net worth context ~$130B.</t>
+          <t>Converted to a family office in 2011, returning ~$25.5B in outside capital to avoid mandatory SEC registration under Dodd-Frank.</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>2025: $283M Barcelona office building (from Blackstone); 49% stake in UK's PD Ports (from Brookfield); $780M Vancouver building (from QuadReal).</t>
-        </is>
-      </c>
-      <c r="S42" t="inlineStr">
-        <is>
-          <t>2025-11-24</t>
-        </is>
-      </c>
+          <t>Recent portfolio emphasis on high-growth technology and scaled industrial exposure (positions in Amazon, NVIDIA, Alphabet per 13F).</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr"/>
       <c r="T42" t="b">
         <v>1</v>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>Spain-based. Described as 'the primary investment vehicle and de facto family office of Amancio Ortega... one of the largest single family offices in Europe by assets'. Very well documented, active 2025 dealflow: $283M Barcelona office building (from Blackstone), 49% stake in UK's PD Ports (from Brookfield), $780M Vancouver building (from QuadReal). Net worth context ~$130B.</t>
+          <t>New York. Converted to a family office in 2011, returning essentially all external investor capital (had been ~$25.5B, returned down to under $1B by year-end) specifically to avoid mandatory SEC investment-adviser registration under Dodd-Frank. 'His firm would focus on managing assets solely for Soros and his family.' Widely and repeatedly covered (InvestmentNews, WealthBriefing, PipelineRoad).</t>
         </is>
       </c>
       <c r="V42" t="n">
@@ -5028,7 +5052,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.caproasia.com/2026/04/26/spain-fashion-zara-founder-billionaire-amancio-ortega-age-90-with-130-billion-fortune-family-office-property-group-pontegadea-bought-more-than-1-5-billion-properties-in-north-america-europe/</t>
+          <t>press_named_sfo: https://www.investmentnews.com/retirement-planning/george-soros-ditches-hedge-fund-empire-for-a-family-office/37776</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
@@ -5038,55 +5062,63 @@
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>Foreign entity, same caveat as Valhalla Ventures - press-verified only, no US SEC/ProPublica cross-check possible.</t>
+          <t>Press/database verified, not SEC-primary verified (though the Dodd-Frank registration-avoidance motive is itself a well-documented regulatory fact, not just a press characterization).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Soros Fund Management</t>
+          <t>Tarbox Family Office, Inc.</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Single-Family Office</t>
+          <t>Multi-Family Office</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>George Soros</t>
+          <t>Laura Tarbox</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Founder</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr"/>
+          <t>Founder (CFP, 1984)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Laura@Tarbox.com</t>
+        </is>
+      </c>
       <c r="F43" t="b">
         <v>0</v>
       </c>
-      <c r="G43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>949-721-2330</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/soros-fund-management</t>
+          <t>https://www.linkedin.com/company/tarboxfamilyoffice</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://sorosfundmgmt.com</t>
+          <t>https://tarbox.com</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Newport Beach</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -5096,49 +5128,53 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>~$28B net assets</t>
+          <t>$1B+</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Reflexivity-theory-informed: investor biases and market fundamentals form feedback loops affecting prices. Unconstrained global mandate across equities, credit, fixed income, macro, and private equity; takes large concentrated positions when conviction is high. Distinctively, the firm's stated primary mandate is to serve as the permanent capital base funding the Open Society Foundations.</t>
+          <t>Evolved from active stock-picking to an evidence-based, tax-efficient, asset-class investing approach using indexed core exposures, controlled diversification, and tax-aware management, with room for alternatives/interval funds when appropriate. Fee-only since 1990 (no commissions/trails/referral fees).</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Equities, credit, fixed income, macro, private equity - technology and industrial exposure</t>
+          <t>Index-based core equity/fixed income exposures, tax-aware; selective alternatives</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>Converted to a family office in 2011, returning ~$25.5B in outside capital to avoid mandatory SEC registration under Dodd-Frank.</t>
+          <t>Founded 1985. Fee-only, 100+ client families.</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Recent portfolio emphasis on high-growth technology and scaled industrial exposure (positions in Amazon, NVIDIA, Alphabet per 13F).</t>
-        </is>
-      </c>
-      <c r="S43" t="inlineStr"/>
+          <t>Most recent 13F filing (2026-04-24) shows a position in Ishares Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
       <c r="T43" t="b">
         <v>1</v>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>New York. Converted to a family office in 2011, returning essentially all external investor capital (had been ~$25.5B, returned down to under $1B by year-end) specifically to avoid mandatory SEC investment-adviser registration under Dodd-Frank. 'His firm would focus on managing assets solely for Soros and his family.' Widely and repeatedly covered (InvestmentNews, WealthBriefing, PipelineRoad).</t>
+          <t>Newport Beach CA, founded 1985 by Laura Tarbox. Explicitly self-described: 'the multi-family office is uniquely positioned with just 100+ client families and over $1 billion under management' - direct, explicit multi-family self-declaration.</t>
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>press_named_sfo</t>
+          <t>own_website</t>
         </is>
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.investmentnews.com/retirement-planning/george-soros-ditches-hedge-fund-empire-for-a-family-office/37776</t>
+          <t>own_website: https://tarbox.com/who-we-are/</t>
         </is>
       </c>
       <c r="Y43" t="inlineStr">
@@ -5148,106 +5184,94 @@
       </c>
       <c r="Z43" t="inlineStr">
         <is>
-          <t>Press/database verified, not SEC-primary verified (though the Dodd-Frank registration-avoidance motive is itself a well-documented regulatory fact, not just a press characterization).</t>
+          <t>13F-HR filer, matched keyword 'family office'. Location: Newport Beach, CA. | Email/phone match firm domain, corroborated by a conference speaker-bio PDF Tarbox herself likely supplied - not deliverability-confirmed.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tarbox Family Office, Inc.</t>
+          <t>The Dalio Family Office</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Multi-Family Office</t>
+          <t>Single-Family Office</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Laura Tarbox</t>
+          <t>Ray Dalio</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Founder (CFP, 1984)</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Laura@Tarbox.com</t>
-        </is>
-      </c>
+          <t>Founder &amp; CIO (Bridgewater Associates founder)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
       <c r="F44" t="b">
         <v>0</v>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>949-721-2330</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/raydalio</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/tarboxfamilyoffice</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>https://tarbox.com</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/dalio-family-office</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Newport Beach</t>
+          <t>Westport</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>USA / UAE / Singapore</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>$1B+</t>
+          <t>~$15B personal wealth</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Evolved from active stock-picking to an evidence-based, tax-efficient, asset-class investing approach using indexed core exposures, controlled diversification, and tax-aware management, with room for alternatives/interval funds when appropriate. Fee-only since 1990 (no commissions/trails/referral fees).</t>
+          <t>Macro-driven allocation informed by Dalio's published views on government debt, US dollar reserve-currency risk, and historical great-power transitions - reflected in a gold-heavy tilt (reported &gt;75% of the office's US stock-adjacent allocation in a gold-tracking ETF) alongside Treasuries and broad equity ETFs. Also runs a growing venture portfolio in AI, fintech, and data analytics. Deploys via direct co-investments, fund commitments, and real-asset holdings.</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Index-based core equity/fixed income exposures, tax-aware; selective alternatives</t>
+          <t>Gold/precious metals, Treasuries, broad equity ETFs, AI/fintech/data-analytics venture portfolio</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>Founded 1985. Fee-only, 100+ client families.</t>
+          <t>Established 2011 to manage Dalio's personal investments and coordinate estate/philanthropic matters following his retirement from Bridgewater. Offices in the US, Abu Dhabi Global Market, and Singapore.</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-04-24) shows a position in Ishares Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
-        </is>
-      </c>
-      <c r="S44" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
+          <t>Mark Baumgartner named as new Investment Chief for the family office (per LinkedIn coverage).</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr"/>
       <c r="T44" t="b">
         <v>1</v>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>Newport Beach CA, founded 1985 by Laura Tarbox. Explicitly self-described: 'the multi-family office is uniquely positioned with just 100+ client families and over $1 billion under management' - direct, explicit multi-family self-declaration.</t>
+          <t>Offices in US, Abu Dhabi Global Market, and Singapore. Established 2011 'to manage the resulting wealth and coordinate estate and philanthropic matters' for Ray Dalio. Following his retirement from Bridgewater, Dalio became CIO of his own family office. Multiply corroborated: Bloomberg ('Ray Dalio Embraces Family Office Life as CIO'), Altss, PipelineRoad, andsimple.co case study.</t>
         </is>
       </c>
       <c r="V44" t="n">
@@ -5255,12 +5279,12 @@
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>own_website</t>
+          <t>multi_source_corroboration</t>
         </is>
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>own_website: https://tarbox.com/who-we-are/</t>
+          <t>multi_source_corroboration: https://www.bloomberg.com/news/articles/2025-09-17/ray-dalio-embraces-family-office-life-as-cio-i-m-the-guy-now</t>
         </is>
       </c>
       <c r="Y44" t="inlineStr">
@@ -5270,14 +5294,14 @@
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>13F-HR filer, matched keyword 'family office'. Location: Newport Beach, CA. | Email/phone match firm domain, corroborated by a conference speaker-bio PDF Tarbox herself likely supplied - not deliverability-confirmed.</t>
+          <t>Press/database verified, not SEC-primary verified.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>The Dalio Family Office</t>
+          <t>Thiel Capital</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5287,12 +5311,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Ray Dalio</t>
+          <t>Peter Thiel</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Founder &amp; CIO (Bridgewater Associates founder)</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -5300,94 +5324,98 @@
         <v>0</v>
       </c>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/raydalio</t>
-        </is>
-      </c>
+      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/dalio-family-office</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/thiel-capital-llc</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://www.thielcapital.com</t>
+        </is>
+      </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Westport</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>USA / UAE / Singapore</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>~$15B personal wealth</t>
+          <t>~$10B</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Macro-driven allocation informed by Dalio's published views on government debt, US dollar reserve-currency risk, and historical great-power transitions - reflected in a gold-heavy tilt (reported &gt;75% of the office's US stock-adjacent allocation in a gold-tracking ETF) alongside Treasuries and broad equity ETFs. Also runs a growing venture portfolio in AI, fintech, and data analytics. Deploys via direct co-investments, fund commitments, and real-asset holdings.</t>
+          <t>Backs startups that escape competition by building monopolies through unique insight, technology, and defensible market positions - prioritizes foundational differentiation over incremental improvement.</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Gold/precious metals, Treasuries, broad equity ETFs, AI/fintech/data-analytics venture portfolio</t>
+          <t>Artificial intelligence, defense/national security technology, biotechnology, financial infrastructure</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>Established 2011 to manage Dalio's personal investments and coordinate estate/philanthropic matters following his retirement from Bridgewater. Offices in the US, Abu Dhabi Global Market, and Singapore.</t>
+          <t>Peter Thiel's family office (Los Angeles, CA / Miami, FL), providing strategic and operational support for his investment initiatives, backing early/growth-stage technology companies often ahead of institutional VC rounds. Founded 2011. Has incubated Founders Fund, Mithril, and Valar Ventures.</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Mark Baumgartner named as new Investment Chief for the family office (per LinkedIn coverage).</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr"/>
+          <t>Listed among most active family offices for 2025 dealmaking per CNBC's Inside Wealth Family Office 15.</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
       <c r="T45" t="b">
         <v>1</v>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>Offices in US, Abu Dhabi Global Market, and Singapore. Established 2011 'to manage the resulting wealth and coordinate estate and philanthropic matters' for Ray Dalio. Following his retirement from Bridgewater, Dalio became CIO of his own family office. Multiply corroborated: Bloomberg ('Ray Dalio Embraces Family Office Life as CIO'), Altss, PipelineRoad, andsimple.co case study.</t>
+          <t>Listed among most active family offices for 2025 dealmaking per CNBC.</t>
         </is>
       </c>
       <c r="V45" t="n">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>multi_source_corroboration</t>
+          <t>press_named_sfo</t>
         </is>
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>multi_source_corroboration: https://www.bloomberg.com/news/articles/2025-09-17/ray-dalio-embraces-family-office-life-as-cio-i-m-the-guy-now</t>
+          <t>press_named_sfo: https://www.cnbc.com/2026/02/12/inside-wealth-family-office-15.html</t>
         </is>
       </c>
       <c r="Y45" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="Z45" t="inlineStr">
         <is>
-          <t>Press/database verified, not SEC-primary verified.</t>
+          <t>Listed among most active family offices for 2025 dealmaking per CNBC. | Also has a Miami, FL presence per sources - Los Angeles used as primary city.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Thiel Capital</t>
+          <t>Tiger Management</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5397,12 +5425,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Peter Thiel</t>
+          <t>Julian Robertson (d. 2022)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -5411,24 +5439,16 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/thiel-capital-llc</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>https://www.thielcapital.com</t>
-        </is>
-      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -5436,42 +5456,30 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>~$10B</t>
-        </is>
-      </c>
+      <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Backs startups that escape competition by building monopolies through unique insight, technology, and defensible market positions - prioritizes foundational differentiation over incremental improvement.</t>
+          <t>Transitioned from hedge fund to family office in March 2000, retaining ~$760M of Robertson's personal wealth. Initially centered on seeding 'Tiger Cub' funds launched by former employees; current portfolio (per 13F) concentrated in two consumer-discretionary holdings (Coupang, Maplebear/Instacart).</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Artificial intelligence, defense/national security technology, biotechnology, financial infrastructure</t>
+          <t>Public equities (consumer discretionary concentration per latest 13F)</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>Peter Thiel's family office (Los Angeles, CA / Miami, FL), providing strategic and operational support for his investment initiatives, backing early/growth-stage technology companies often ahead of institutional VC rounds. Founded 2011. Has incubated Founders Fund, Mithril, and Valar Ventures.</t>
-        </is>
-      </c>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>Listed among most active family offices for 2025 dealmaking per CNBC's Inside Wealth Family Office 15.</t>
-        </is>
-      </c>
-      <c r="S46" t="inlineStr">
-        <is>
-          <t>2026-02-12</t>
-        </is>
-      </c>
+          <t>Converted from hedge fund to Robertson's own family office. Distinct from the 'Tiger Cubs' - former employees who founded their own separate hedge funds (Lone Pine, Maverick, etc.).</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
       <c r="T46" t="b">
         <v>1</v>
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>Listed among most active family offices for 2025 dealmaking per CNBC.</t>
+          <t>New York. After closing Tiger Management as a hedge fund, Julian Robertson 'converted it into his own family office.' Well documented on Wikipedia and multiple financial history sources. Distinct from the 'Tiger Cubs' - former Tiger employees who founded their OWN separate hedge funds (Lone Pine, Maverick, etc.) - those are NOT part of this entity and should not be conflated with it.</t>
         </is>
       </c>
       <c r="V46" t="n">
@@ -5484,24 +5492,24 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.cnbc.com/2026/02/12/inside-wealth-family-office-15.html</t>
+          <t>press_named_sfo: https://en.wikipedia.org/wiki/Tiger_Management</t>
         </is>
       </c>
       <c r="Y46" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
-          <t>Listed among most active family offices for 2025 dealmaking per CNBC. | Also has a Miami, FL presence per sources - Los Angeles used as primary city.</t>
+          <t>Press/Wikipedia verified, not SEC-primary verified. | Julian Robertson died August 2022. Current (2026) day-to-day leadership/management of the family office post-Robertson was NOT confirmed in sources reviewed - honest gap, not filled with a guess.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tiger Management</t>
+          <t>Valhalla Ventures</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5511,12 +5519,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Julian Robertson (d. 2022)</t>
+          <t>Mark O'Hare</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>Founder (Preqin founder)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -5526,46 +5534,50 @@
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://valhallaventures.co.uk</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Transitioned from hedge fund to family office in March 2000, retaining ~$760M of Robertson's personal wealth. Initially centered on seeding 'Tiger Cub' funds launched by former employees; current portfolio (per 13F) concentrated in two consumer-discretionary holdings (Coupang, Maplebear/Instacart).</t>
+          <t>Patient, long-term capital deployment with no fixed exit horizon; ~70% of the portfolio allocated outside public markets, with an emphasis on secondaries and private credit.</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>Public equities (consumer discretionary concentration per latest 13F)</t>
+          <t>Secondaries, private credit (~70% of portfolio outside public markets)</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>Converted from hedge fund to Robertson's own family office. Distinct from the 'Tiger Cubs' - former employees who founded their own separate hedge funds (Lone Pine, Maverick, etc.).</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
+          <t>O'Hare family holding company for investment and philanthropic activities. Received ~$2.6B from the 2025 Preqin/BlackRock sale.</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Accumulated a 7.2% stake (~$200M) in HgCapital Trust Plc.</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
       <c r="T47" t="b">
         <v>1</v>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>New York. After closing Tiger Management as a hedge fund, Julian Robertson 'converted it into his own family office.' Well documented on Wikipedia and multiple financial history sources. Distinct from the 'Tiger Cubs' - former Tiger employees who founded their OWN separate hedge funds (Lone Pine, Maverick, etc.) - those are NOT part of this entity and should not be conflated with it.</t>
+          <t>UK-based. Press: 'the O'Hare family's holding company managing the family's investment and philanthropic activities'. Sold Preqin to BlackRock (completed ~March 2025) for ~$2.6B to the family. Actively deployed: ~$200M / 7.2% stake in HgCapital Trust Plc, ~70% of portfolio allocated outside public markets.</t>
         </is>
       </c>
       <c r="V47" t="n">
@@ -5578,7 +5590,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://en.wikipedia.org/wiki/Tiger_Management</t>
+          <t>press_named_sfo: https://www.bloomberg.com/news/articles/2026-02-20/billionaire-preqin-seller-s-family-office-builds-buyout-firm-bet</t>
         </is>
       </c>
       <c r="Y47" t="inlineStr">
@@ -5588,14 +5600,14 @@
       </c>
       <c r="Z47" t="inlineStr">
         <is>
-          <t>Press/Wikipedia verified, not SEC-primary verified. | Julian Robertson died August 2022. Current (2026) day-to-day leadership/management of the family office post-Robertson was NOT confirmed in sources reviewed - honest gap, not filled with a guess.</t>
+          <t>UK entity - our SEC 13F/EDGAR and ProPublica 990 tools only cover US filers, so this record is press-verified only, not cross-checked against a primary regulatory filing the way the US SFOs in this dataset are. State this limitation honestly if this record makes the final 50 - do not present it with the same verification depth as e.g. Duquesne or West Family Investments.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Valhalla Ventures</t>
+          <t>Waycrosse, Inc.</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5605,12 +5617,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mark O'Hare</t>
+          <t>Lucy MacMillan Stitzer</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Founder (Preqin founder)</t>
+          <t>Chairman</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -5620,63 +5632,63 @@
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>https://valhallaventures.co.uk</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Wayzata</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr"/>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>~$65B</t>
+        </is>
+      </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Patient, long-term capital deployment with no fixed exit horizon; ~70% of the portfolio allocated outside public markets, with an emphasis on secondaries and private credit.</t>
+          <t>Diversified institutional-style allocation across private equity, private credit, real assets, hedge funds, infrastructure, and insurance-linked strategies.</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>Secondaries, private credit (~70% of portfolio outside public markets)</t>
+          <t>Private equity, private credit, real assets, hedge funds, infrastructure, insurance-linked strategies</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>O'Hare family holding company for investment and philanthropic activities. Received ~$2.6B from the 2025 Preqin/BlackRock sale.</t>
-        </is>
-      </c>
-      <c r="R48" t="inlineStr">
-        <is>
-          <t>Accumulated a 7.2% stake (~$200M) in HgCapital Trust Plc.</t>
-        </is>
-      </c>
-      <c r="S48" t="inlineStr">
-        <is>
-          <t>2026-02-20</t>
-        </is>
-      </c>
+          <t>Founded 1991 to serve the intermarried Cargill and MacMillan families (wealth from Cargill, Incorporated).</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
       <c r="T48" t="b">
         <v>1</v>
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>UK-based. Press: 'the O'Hare family's holding company managing the family's investment and philanthropic activities'. Sold Preqin to BlackRock (completed ~March 2025) for ~$2.6B to the family. Actively deployed: ~$200M / 7.2% stake in HgCapital Trust Plc, ~70% of portfolio allocated outside public markets.</t>
+          <t>Wayzata MN, founded 1991. Directly and explicitly described as 'the single family office for the Cargill-MacMillan families of Minnesota' across multiple independent sources (PipelineRoad, Altss, Forbes profile, Wikipedia entries for Cargill MacMillan Sr./Jr.). ~$65B AUM. Two surnames (Cargill, MacMillan) reflects one intermarried family lineage, not two unrelated families being served as separate clients - consistent with SEC family office rule's lineage definition. Chairman: Lucy MacMillan Stitzer.</t>
         </is>
       </c>
       <c r="V48" t="n">
-        <v>0.4</v>
+        <v>0.65</v>
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>press_named_sfo</t>
+          <t>press_named_sfo, multi_source_corroboration</t>
         </is>
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://www.bloomberg.com/news/articles/2026-02-20/billionaire-preqin-seller-s-family-office-builds-buyout-firm-bet</t>
+          <t>press_named_sfo: https://pipelineroad.com/directory/cargill-macmillan | multi_source_corroboration: https://www.forbes.com/profile/cargill-macmillan-1/</t>
         </is>
       </c>
       <c r="Y48" t="inlineStr">
@@ -5686,14 +5698,14 @@
       </c>
       <c r="Z48" t="inlineStr">
         <is>
-          <t>UK entity - our SEC 13F/EDGAR and ProPublica 990 tools only cover US filers, so this record is press-verified only, not cross-checked against a primary regulatory filing the way the US SFOs in this dataset are. State this limitation honestly if this record makes the final 50 - do not present it with the same verification depth as e.g. Duquesne or West Family Investments.</t>
+          <t>No SEC 13F/ADV filing found under this name despite large AUM - likely invests via external managers rather than filing directly. Press/multi-source verified, not SEC-primary verified. | No public official website found - consistent with the Cargill family's well-documented preference for low public visibility. Honest gap, not an oversight.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Waycrosse, Inc.</t>
+          <t>West Family Investments, Inc.</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5703,12 +5715,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Lucy MacMillan Stitzer</t>
+          <t>Gary West</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Chairman</t>
+          <t>Managing Principal (with Mary West)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -5721,12 +5733,12 @@
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Wayzata</t>
+          <t>Carlsbad</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -5736,45 +5748,53 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>~$65B</t>
+          <t>$383M in 13F-reportable securities (Q2 2025), 366 equity positions, largest holding iShares Gold Trust</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Diversified institutional-style allocation across private equity, private credit, real assets, hedge funds, infrastructure, and insurance-linked strategies.</t>
+          <t>Combines rigorous financial/market analysis with a network-driven approach to identify innovative, sector-leading companies. Notable healthcare innovation focus via the $100M West Health Investment Fund (risk capital for cost-lowering healthcare technology). West Partners (the PE arm) makes $10-100M control investments in private companies plus commercial real estate.</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>Private equity, private credit, real assets, hedge funds, infrastructure, insurance-linked strategies</t>
+          <t>Healthcare innovation, private equity control investments, commercial real estate</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>Founded 1991 to serve the intermarried Cargill and MacMillan families (wealth from Cargill, Incorporated).</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
+          <t>Gary and Mary West's single-family office (Carlsbad, CA), SEC-confirmed as exempt under the Family Office Exemption. Known for healthcare-innovation investing and West Partners, its private-equity/real-estate arm.</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Most recent 13F filing (2026-05-07) shows a position in Ishares Gold Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
       <c r="T49" t="b">
         <v>1</v>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>Wayzata MN, founded 1991. Directly and explicitly described as 'the single family office for the Cargill-MacMillan families of Minnesota' across multiple independent sources (PipelineRoad, Altss, Forbes profile, Wikipedia entries for Cargill MacMillan Sr./Jr.). ~$65B AUM. Two surnames (Cargill, MacMillan) reflects one intermarried family lineage, not two unrelated families being served as separate clients - consistent with SEC family office rule's lineage definition. Chairman: Lucy MacMillan Stitzer.</t>
+          <t>Carlsbad CA, principals Gary and Mary West. PRIMARY SOURCE: SEC Schedule 13D/13G filing states directly: 'The Adviser is a family office exempt from registration under the Family Office Exemption.' Continuously active 2013-2026 (97 filings).</t>
         </is>
       </c>
       <c r="V49" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>press_named_sfo, multi_source_corroboration</t>
+          <t>sec_primary_declaration, sec_13f_clean</t>
         </is>
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://pipelineroad.com/directory/cargill-macmillan | multi_source_corroboration: https://www.forbes.com/profile/cargill-macmillan-1/</t>
+          <t>sec_primary_declaration: https://www.sec.gov/Archives/edgar/data/1568303/0001104659-21-108534.txt</t>
         </is>
       </c>
       <c r="Y49" t="inlineStr">
@@ -5784,14 +5804,14 @@
       </c>
       <c r="Z49" t="inlineStr">
         <is>
-          <t>No SEC 13F/ADV filing found under this name despite large AUM - likely invests via external managers rather than filing directly. Press/multi-source verified, not SEC-primary verified. | No public official website found - consistent with the Cargill family's well-documented preference for low public visibility. Honest gap, not an oversight.</t>
+          <t>13F-HR filer, matched keyword 'family investments'. Location: Evanston, IL. | A LinkedIn profile for a 'Gary West' at 'Gary West Investments LLC' surfaced but the entity name doesn't clearly match West Family Investments, Inc. - not used as principal_linkedin to avoid a wrong-person/wrong-entity error. | One aggregator (Bloomberg profile) listed Evanston, IL as a location, contradicting all other sources (SEC filing, primary research) which consistently show Carlsbad, CA - treated as aggregator error, Carlsbad retained.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>West Family Investments, Inc.</t>
+          <t>Wildcat Capital Management</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5801,12 +5821,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Gary West</t>
+          <t>David Bonderman (d. Dec 2024); Len Potter (CEO &amp; CIO, operating principal)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Managing Principal (with Mary West)</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -5815,51 +5835,47 @@
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Carlsbad</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/wildcat-capital-management</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://www.wildcatcap.com</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
-          <t>$383M in 13F-reportable securities (Q2 2025), 366 equity positions, largest holding iShares Gold Trust</t>
+          <t>$4.08-4.1B</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Combines rigorous financial/market analysis with a network-driven approach to identify innovative, sector-leading companies. Notable healthcare innovation focus via the $100M West Health Investment Fund (risk capital for cost-lowering healthcare technology). West Partners (the PE arm) makes $10-100M control investments in private companies plus commercial real estate.</t>
+          <t>Public equities and direct investments; measured, long-term positioning rather than rapid trading (e.g. the TIC Solutions exit was a multi-year hold).</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>Healthcare innovation, private equity control investments, commercial real estate</t>
+          <t>Public equities, direct investments</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>Gary and Mary West's single-family office (Carlsbad, CA), SEC-confirmed as exempt under the Family Office Exemption. Known for healthcare-innovation investing and West Partners, its private-equity/real-estate arm.</t>
+          <t>Founded 2011 as the single-family office of David Bonderman, TPG co-founder.</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Most recent 13F filing (2026-05-07) shows a position in Ishares Gold Tr. Reported position VALUE not cited here - cross-check against this firm's own AUM found it implausibly large (same pattern as the Kemnay/West Family Investments unit-reliability issue documented elsewhere in this project), so only the holding name and filing date are used as the verified signal.</t>
+          <t>Sold 1.5 million shares of TIC Solutions in Q3 2025, worth an estimated $16.56 million.</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2025-12-26</t>
         </is>
       </c>
       <c r="T50" t="b">
@@ -5867,37 +5883,37 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>Carlsbad CA, principals Gary and Mary West. PRIMARY SOURCE: SEC Schedule 13D/13G filing states directly: 'The Adviser is a family office exempt from registration under the Family Office Exemption.' Continuously active 2013-2026 (97 filings).</t>
+          <t>Founded 2011 as single-family office; recent $16.6M exit from TIC Solutions covered by Motley Fool/Yahoo Finance.</t>
         </is>
       </c>
       <c r="V50" t="n">
-        <v>0.75</v>
+        <v>0.4</v>
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>sec_primary_declaration, sec_13f_clean</t>
+          <t>press_named_sfo</t>
         </is>
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>sec_primary_declaration: https://www.sec.gov/Archives/edgar/data/1568303/0001104659-21-108534.txt</t>
+          <t>press_named_sfo: https://finance.yahoo.com/news/billionaire-family-offices-16-6-183153119.html</t>
         </is>
       </c>
       <c r="Y50" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="Z50" t="inlineStr">
         <is>
-          <t>13F-HR filer, matched keyword 'family investments'. Location: Evanston, IL. | A LinkedIn profile for a 'Gary West' at 'Gary West Investments LLC' surfaced but the entity name doesn't clearly match West Family Investments, Inc. - not used as principal_linkedin to avoid a wrong-person/wrong-entity error. | One aggregator (Bloomberg profile) listed Evanston, IL as a location, contradicting all other sources (SEC filing, primary research) which consistently show Carlsbad, CA - treated as aggregator error, Carlsbad retained.</t>
+          <t>Founded 2011 as single-family office; recent $16.6M exit from TIC Solutions covered by Motley Fool/Yahoo Finance. | CAVEAT: one source describes Wildcat as also 'managing assets for an institutional client base' beyond the Bonderman family - worth a closer look before treating single-family status as beyond question, though the original press evidence (explicit 'founded as the single-family office of David Bonderman') remains solid. | Len Potter (ex-Soros Fund Management PE co-head) founded/runs Wildcat as CEO &amp; CIO since 2011 - the OPERATING principal, distinct from David Bonderman as the family principal whose wealth the office manages. Both are legitimately 'principals' in different senses. | General office contact found on firm website (wildcatcap.com), NOT verified as a principal's direct line: info@wildcatcap.com, 212-468-5100, 888 7th Avenue 37th Fl, New York, NY 10106.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Wildcat Capital Management</t>
+          <t>Willett Advisors LLC</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5907,7 +5923,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>David Bonderman (d. Dec 2024); Len Potter (CEO &amp; CIO, operating principal)</t>
+          <t>Michael Bloomberg (family principal); Steven Rattner (Chairman &amp; CEO, operating principal)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5923,45 +5939,49 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/wildcat-capital-management</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>https://www.wildcatcap.com</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>$4.08-4.1B</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/willett-advisors-llc</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Public equities and direct investments; measured, long-term positioning rather than rapid trading (e.g. the TIC Solutions exit was a multi-year hold).</t>
+          <t>Long-term capital appreciation via a diversified multi-asset-class portfolio; deploys through direct investments and select third-party managers across public markets, private equity/credit, hedge funds, real assets, and direct venture investments.</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Public equities, direct investments</t>
+          <t>Public markets, private equity/credit, hedge funds, real assets, venture (growth/late-stage)</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>Founded 2011 as the single-family office of David Bonderman, TPG co-founder.</t>
+          <t>Single-family office of Michael R. Bloomberg, founded 2010. Manages Bloomberg's personal and philanthropic assets, integrating investment returns with Bloomberg Philanthropies' mission across education, public health, and environment.</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Sold 1.5 million shares of TIC Solutions in Q3 2025, worth an estimated $16.56 million.</t>
+          <t>Participated in Cellares' Series D financing (announced $257M January 2026, expanded to $327M June 2026). 16 total investments as of early 2026, focused on growth/late-stage rounds (Series B/C); portfolio includes Circle and Finch Therapeutics.</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="T51" t="b">
@@ -5969,30 +5989,30 @@
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>Founded 2011 as single-family office; recent $16.6M exit from TIC Solutions covered by Motley Fool/Yahoo Finance.</t>
+          <t>Established 2010 as the single-family office of Michael R. Bloomberg (Bloomberg L.P. founder, former NYC Mayor). Confirmed via SEC EDGAR (CIK 1509379, registered NYC entity, address matches independent sources exactly) and multiple independent press/reference sources (Wikipedia's dedicated 'Willett Advisors' article, familyofficehub.io, PipelineRoad) explicitly and unambiguously describing it as Bloomberg's family office - no name-collision risk of the kind that disqualified a previous candidate record in this dataset.</t>
         </is>
       </c>
       <c r="V51" t="n">
-        <v>0.4</v>
+        <v>0.75</v>
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>press_named_sfo</t>
+          <t>press_named_sfo, sec_filing</t>
         </is>
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>press_named_sfo: https://finance.yahoo.com/news/billionaire-family-offices-16-6-183153119.html</t>
+          <t>press_named_sfo: https://en.wikipedia.org/wiki/Willett_Advisors | sec_filing: https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001509379&amp;type=13F-HR</t>
         </is>
       </c>
       <c r="Y51" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="Z51" t="inlineStr">
         <is>
-          <t>Founded 2011 as single-family office; recent $16.6M exit from TIC Solutions covered by Motley Fool/Yahoo Finance. | CAVEAT: one source describes Wildcat as also 'managing assets for an institutional client base' beyond the Bonderman family - worth a closer look before treating single-family status as beyond question, though the original press evidence (explicit 'founded as the single-family office of David Bonderman') remains solid. | Len Potter (ex-Soros Fund Management PE co-head) founded/runs Wildcat as CEO &amp; CIO since 2011 - the OPERATING principal, distinct from David Bonderman as the family principal whose wealth the office manages. Both are legitimately 'principals' in different senses. | General office contact found on firm website (wildcatcap.com), NOT verified as a principal's direct line: info@wildcatcap.com, 212-468-5100, 888 7th Avenue 37th Fl, New York, NY 10106.</t>
+          <t>SEC 13F filings for this entity (CIK 1509379) are stale - last filed 2014, over a decade ago. Used as source class 'sec_filing' (confirms the entity is real and registered) rather than 'sec_13f_clean' (which specifically means current filing activity) - a deliberate distinction, not an oversight. Minor address discrepancy noted, not reconciled: SEC's registered address is 650 Madison Avenue, NY; one LinkedIn/directory source lists 25 E 78th St, NY - both in Manhattan. AUM left honestly blank - no figure found with a confidence-worthy source this session.</t>
         </is>
       </c>
     </row>

</xml_diff>